<commit_message>
Popraw opisy oceny ryzyka dla scenariuszy EPU nakaz zapłaty (24 wiersze)
- EPU_NAKAZ_SPOLKA: wyjaśnienie mechanizmu art. 299 KSH z uwzględnieniem
  specyfiki EPU (sprzeciw elektroniczny, przeniesienie do sądu zwykłego)
- EPU_NAKAZ_CZLONEK_ZARZADU: odpowiedzialność osobista + EPU sprzeciw
  uproszczony ale obowiązkowy w terminie
- Teksty różnicowane wg risk_level (URGENT/HIGH/MEDIUM/LOW)
- CSV i Excel zsynchronizowane

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -4526,12 +4526,12 @@
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>Podwyższona pilność wynika przede wszystkim z rodzaju dokumentu oraz możliwego biegu terminu na reakcję. Czas na reakcję może być ograniczony, dlatego kluczowe jest potwierdzenie daty doręczenia i treści pouczenia. Brak pełnych dokumentów ogranicza pewność wstępnej oceny. Ponieważ dokument może pochodzić z EPU/e-Sądu, trzeba odrębnie sprawdzić właściwy tryb i termin reakcji. Ponieważ dokument wskazuje na e-Sąd (EPU), priorytetem jest szybkie zabezpieczenie reakcji w terminie, a pełna strategia i materiał dowodowy mogą zostać dopracowane w kolejnym etapie po przekazaniu sprawy do sądu właściwości ogólnej.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS. Ponieważ dokument wskazuje na e-Sąd (EPU), priorytetem jest szybkie zabezpieczenie reakcji w terminie, a pełna strategia i materiał dowodowy mogą zostać dopracowane w kolejnym etapie po przekazaniu sprawy do sądu właściwości ogólnej.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P28" s="5" t="inlineStr">
@@ -4641,12 +4641,12 @@
       </c>
       <c r="N29" s="5" t="inlineStr">
         <is>
-          <t>Wysokie ryzyko wynika z połączenia rodzaju dokumentu, potrzeby weryfikacji terminu oraz niepewności danych wymagających sprawdzenia. Czas na reakcję może być ograniczony, dlatego kluczowe jest potwierdzenie daty doręczenia i treści pouczenia. Dosłanie dokumentów może istotnie zmienić szczegółową ocenę sprawy. Ponieważ dokument może pochodzić z EPU/e-Sądu, trzeba odrębnie sprawdzić właściwy tryb i termin reakcji. Możesz zacząć od wstępnej oceny, a dokumenty dosłać później — plan ułożymy etapowo.</t>
+          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie jako członka zarządu. Masz jeszcze czas na złożenie sprzeciwu w EPU, ale wymaga to weryfikacji: daty doręczenia, treści pouczenia oraz podstawy roszczenia. W EPU sprzeciw może być początkowo uproszczony — ważne jest złożenie go w terminie.</t>
         </is>
       </c>
       <c r="O29" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P29" s="5" t="inlineStr">
@@ -4756,12 +4756,12 @@
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>Podwyższona pilność wynika przede wszystkim z rodzaju dokumentu oraz możliwego biegu terminu na reakcję. Czas na reakcję może być ograniczony, dlatego kluczowe jest potwierdzenie daty doręczenia i treści pouczenia. Dosłanie dokumentów może istotnie zmienić szczegółową ocenę sprawy. Status rezygnacji lub odwołania oraz aktualność wpisu w KRS wymagają weryfikacji. Ponieważ dokument może pochodzić z EPU/e-Sądu, trzeba odrębnie sprawdzić właściwy tryb i termin reakcji. Ponieważ dokument pochodzi z e-Sądu, zakres czynności na etapie samej reakcji terminowej może być organizacyjnie prostszy, ale równolegle należy przygotować plan dalszej obrony na etap po przekazaniu sprawy do sądu właściwego.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
         </is>
       </c>
       <c r="O30" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS. Ponieważ dokument pochodzi z e-Sądu, zakres czynności na etapie samej reakcji terminowej może być organizacyjnie prostszy, ale równolegle należy przygotować plan dalszej obrony na etap po przekazaniu sprawy do sądu właściwego.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P30" s="5" t="inlineStr">
@@ -4867,12 +4867,12 @@
       </c>
       <c r="N31" s="5" t="inlineStr">
         <is>
-          <t>Wysokie ryzyko wynika z połączenia rodzaju dokumentu, potrzeby weryfikacji terminu oraz niepewności danych wymagających sprawdzenia. Ponieważ dokument może pochodzić z EPU/e-Sądu, trzeba odrębnie sprawdzić właściwy tryb i termin reakcji. W przypadku e-Sądu rekomendowany jest Audyt 48h skoncentrowany na prawidłowej organizacji reakcji terminowej oraz przygotowaniu dalszej strategii na etap po ewentualnym przekazaniu sprawy do sądu właściwego.</t>
+          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie jako członka zarządu. Masz jeszcze czas na złożenie sprzeciwu w EPU, ale wymaga to weryfikacji: daty doręczenia, treści pouczenia oraz podstawy roszczenia. W EPU sprzeciw może być początkowo uproszczony — ważne jest złożenie go w terminie.</t>
         </is>
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS. W przypadku e-Sądu rekomendowany jest Audyt 48h skoncentrowany na prawidłowej organizacji reakcji terminowej oraz przygotowaniu dalszej strategii na etap po ewentualnym przekazaniu sprawy do sądu właściwego.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P31" s="5" t="inlineStr">
@@ -4978,12 +4978,12 @@
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>Ryzyko oceniono jako średnie, ale wynik nadal wymaga weryfikacji dokumentów i terminów. Ponieważ dokument może pochodzić z EPU/e-Sądu, trzeba odrębnie sprawdzić właściwy tryb i termin reakcji.</t>
+          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie. Ryzyko jest ocenione jako umiarkowane — warto jednak potwierdzić termin i podstawę roszczenia przed podjęciem decyzji o złożeniu sprzeciwu w EPU.</t>
         </is>
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P32" s="5" t="inlineStr">
@@ -5089,12 +5089,12 @@
       </c>
       <c r="N33" s="5" t="inlineStr">
         <is>
-          <t>Podwyższona pilność wynika przede wszystkim z rodzaju dokumentu oraz możliwego biegu terminu na reakcję. Brak pełnych dokumentów ogranicza pewność wstępnej oceny. Ponieważ dokument może pochodzić z EPU/e-Sądu, trzeba odrębnie sprawdzić właściwy tryb i termin reakcji. Na tym etapie deklarujesz wstępną ocenę bez wysyłki dokumentów, więc rekomendacja ma charakter organizacyjny i zaczyna od ustalenia braków.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
         </is>
       </c>
       <c r="O33" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P33" s="5" t="inlineStr">
@@ -5200,12 +5200,12 @@
       </c>
       <c r="N34" s="5" t="inlineStr">
         <is>
-          <t>Wysokie ryzyko wynika z połączenia rodzaju dokumentu, potrzeby weryfikacji terminu oraz niepewności danych wymagających sprawdzenia. Brak pełnych dokumentów ogranicza pewność wstępnej oceny. Ponieważ dokument może pochodzić z EPU/e-Sądu, trzeba odrębnie sprawdzić właściwy tryb i termin reakcji. Masz ponad 2 tygodnie na reakcję — można działać spokojniej, ale warto od razu ustalić plan i checklistę.</t>
+          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie jako członka zarządu. Masz jeszcze czas na złożenie sprzeciwu w EPU, ale wymaga to weryfikacji: daty doręczenia, treści pouczenia oraz podstawy roszczenia. W EPU sprzeciw może być początkowo uproszczony — ważne jest złożenie go w terminie.</t>
         </is>
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P34" s="5" t="inlineStr">
@@ -5311,12 +5311,12 @@
       </c>
       <c r="N35" s="5" t="inlineStr">
         <is>
-          <t>Ryzyko oceniono jako średnie, ale wynik nadal wymaga weryfikacji dokumentów i terminów. Dosłanie dokumentów może istotnie zmienić szczegółową ocenę sprawy. Ponieważ dokument może pochodzić z EPU/e-Sądu, trzeba odrębnie sprawdzić właściwy tryb i termin reakcji. Masz ponad 2 tygodnie na reakcję — można działać spokojniej, ale warto od razu ustalić plan i checklistę.</t>
+          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie. Ryzyko jest ocenione jako umiarkowane — warto jednak potwierdzić termin i podstawę roszczenia przed podjęciem decyzji o złożeniu sprzeciwu w EPU.</t>
         </is>
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr">
@@ -5422,12 +5422,12 @@
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>Podwyższona pilność wynika przede wszystkim z rodzaju dokumentu oraz możliwego biegu terminu na reakcję. Brak pełnych dokumentów ogranicza pewność wstępnej oceny. Ponieważ dokument może pochodzić z EPU/e-Sądu, trzeba odrębnie sprawdzić właściwy tryb i termin reakcji. Masz ponad 2 tygodnie na reakcję — można działać spokojniej, ale warto od razu ustalić plan i checklistę.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
         </is>
       </c>
       <c r="O36" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P36" s="5" t="inlineStr">
@@ -5537,12 +5537,12 @@
       </c>
       <c r="N37" s="5" t="inlineStr">
         <is>
-          <t>Wysokie ryzyko wynika z połączenia rodzaju dokumentu, potrzeby weryfikacji terminu oraz niepewności danych wymagających sprawdzenia. Nieustalony termin zwiększa niepewność i wymaga sprawdzenia przed podjęciem dalszych decyzji. Dosłanie dokumentów może istotnie zmienić szczegółową ocenę sprawy. Ponieważ dokument może pochodzić z EPU/e-Sądu, trzeba odrębnie sprawdzić właściwy tryb i termin reakcji. Możesz zacząć od wstępnej oceny, a dokumenty dosłać później — plan ułożymy etapowo.</t>
+          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie jako członka zarządu. Masz jeszcze czas na złożenie sprzeciwu w EPU, ale wymaga to weryfikacji: daty doręczenia, treści pouczenia oraz podstawy roszczenia. W EPU sprzeciw może być początkowo uproszczony — ważne jest złożenie go w terminie.</t>
         </is>
       </c>
       <c r="O37" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P37" s="5" t="inlineStr">
@@ -5652,12 +5652,12 @@
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>Podwyższona pilność wynika przede wszystkim z rodzaju dokumentu oraz możliwego biegu terminu na reakcję. Nieustalony termin zwiększa niepewność i wymaga sprawdzenia przed podjęciem dalszych decyzji. Brak pełnych dokumentów ogranicza pewność wstępnej oceny. Ponieważ dokument może pochodzić z EPU/e-Sądu, trzeba odrębnie sprawdzić właściwy tryb i termin reakcji. Na tym etapie deklarujesz wstępną ocenę bez wysyłki dokumentów, więc rekomendacja ma charakter organizacyjny i zaczyna od ustalenia braków.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
         </is>
       </c>
       <c r="O38" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P38" s="5" t="inlineStr">
@@ -5763,12 +5763,12 @@
       </c>
       <c r="N39" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ nakaz EPU może uruchamiać termin na reakcję, a czas może być krótki albo dane mogą wymagać szybkiego potwierdzenia. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce stwarza bezpośrednie ryzyko dla członka zarządu — jeśli spółka nie złoży sprzeciwu w EPU w terminie, nakaz się uprawomocni. Wierzyciel uruchomi egzekucję, a po jej bezskuteczności skieruje roszczenie bezpośrednio do Ciebie z art. 299 KSH. W EPU termin na sprzeciw jest ściśle liczony od doręczenia — pilność wynika z krótkiego czasu i wymogów elektronicznego postępowania.</t>
         </is>
       </c>
       <c r="O39" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P39" s="5" t="inlineStr">
@@ -5870,12 +5870,12 @@
       </c>
       <c r="N40" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji. Nakaz przeciwko spółce nie zawsze jest dokumentem bezpośrednio skierowanym do członka zarządu, ale może być ważny dla oceny ryzyka odpowiedzialności członka zarządu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce może w konsekwencji prowadzić do osobistej odpowiedzialności członka zarządu z art. 299 KSH — jeśli egzekucja przeciwko spółce okaże się bezskuteczna. Masz jeszcze czas na weryfikację, ale termin na sprzeciw spółki w EPU jest ściśle określony i liczony od doręczenia.</t>
         </is>
       </c>
       <c r="O40" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P40" s="5" t="inlineStr">
@@ -5977,12 +5977,12 @@
       </c>
       <c r="N41" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ nakaz EPU może uruchamiać termin na reakcję, a czas może być krótki albo dane mogą wymagać szybkiego potwierdzenia. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce stwarza bezpośrednie ryzyko dla członka zarządu — jeśli spółka nie złoży sprzeciwu w EPU w terminie, nakaz się uprawomocni. Wierzyciel uruchomi egzekucję, a po jej bezskuteczności skieruje roszczenie bezpośrednio do Ciebie z art. 299 KSH. W EPU termin na sprzeciw jest ściśle liczony od doręczenia — pilność wynika z krótkiego czasu i wymogów elektronicznego postępowania.</t>
         </is>
       </c>
       <c r="O41" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P41" s="5" t="inlineStr">
@@ -6084,12 +6084,12 @@
       </c>
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji. Nakaz przeciwko spółce nie zawsze jest dokumentem bezpośrednio skierowanym do członka zarządu, ale może być ważny dla oceny ryzyka odpowiedzialności członka zarządu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce może w konsekwencji prowadzić do osobistej odpowiedzialności członka zarządu z art. 299 KSH — jeśli egzekucja przeciwko spółce okaże się bezskuteczna. Masz jeszcze czas na weryfikację, ale termin na sprzeciw spółki w EPU jest ściśle określony i liczony od doręczenia.</t>
         </is>
       </c>
       <c r="O42" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P42" s="5" t="inlineStr">
@@ -6191,12 +6191,12 @@
       </c>
       <c r="N43" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji. Nakaz EPU przeciwko spółce może być istotny jako dokument pokazujący etap sprawy, ale sam w sobie nie musi jeszcze oznaczać dokumentu bezpośrednio skierowanego do członka zarządu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU przeciwko spółce wymaga sprawdzenia, czy spółka podjęła już działania. W EPU brak sprzeciwu w terminie powoduje uprawomocnienie nakazu i może w przyszłości przełożyć się na ryzyko z art. 299 KSH dla członka zarządu.</t>
         </is>
       </c>
       <c r="O43" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P43" s="5" t="inlineStr">
@@ -6298,12 +6298,12 @@
       </c>
       <c r="N44" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ nakaz EPU może uruchamiać termin na reakcję, a czas może być krótki albo dane mogą wymagać szybkiego potwierdzenia. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce stwarza bezpośrednie ryzyko dla członka zarządu — jeśli spółka nie złoży sprzeciwu w EPU w terminie, nakaz się uprawomocni. Wierzyciel uruchomi egzekucję, a po jej bezskuteczności skieruje roszczenie bezpośrednio do Ciebie z art. 299 KSH. W EPU termin na sprzeciw jest ściśle liczony od doręczenia — pilność wynika z krótkiego czasu i wymogów elektronicznego postępowania.</t>
         </is>
       </c>
       <c r="O44" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P44" s="5" t="inlineStr">
@@ -6405,12 +6405,12 @@
       </c>
       <c r="N45" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji. Nakaz przeciwko spółce nie zawsze jest dokumentem bezpośrednio skierowanym do członka zarządu, ale może być ważny dla oceny ryzyka odpowiedzialności członka zarządu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce może w konsekwencji prowadzić do osobistej odpowiedzialności członka zarządu z art. 299 KSH — jeśli egzekucja przeciwko spółce okaże się bezskuteczna. Masz jeszcze czas na weryfikację, ale termin na sprzeciw spółki w EPU jest ściśle określony i liczony od doręczenia.</t>
         </is>
       </c>
       <c r="O45" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P45" s="5" t="inlineStr">
@@ -6512,12 +6512,12 @@
       </c>
       <c r="N46" s="5" t="inlineStr">
         <is>
-          <t>Sprawa ma niższy poziom pilności, ale nadal warto potwierdzić podstawowe dane, zwłaszcza termin i adresata nakazu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU przeciwko spółce jest na tym etapie oceniany jako niskie ryzyko bezpośrednie. Warto jednak potwierdzić, czy spółka złożyła sprzeciw w EPU w terminie — brak reakcji mógłby w przyszłości prowadzić do ryzyka z art. 299 KSH dla członka zarządu.</t>
         </is>
       </c>
       <c r="O46" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P46" s="5" t="inlineStr">
@@ -6619,12 +6619,12 @@
       </c>
       <c r="N47" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji. Nakaz EPU przeciwko spółce może być istotny jako dokument pokazujący etap sprawy, ale sam w sobie nie musi jeszcze oznaczać dokumentu bezpośrednio skierowanego do członka zarządu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU przeciwko spółce wymaga sprawdzenia, czy spółka podjęła już działania. W EPU brak sprzeciwu w terminie powoduje uprawomocnienie nakazu i może w przyszłości przełożyć się na ryzyko z art. 299 KSH dla członka zarządu.</t>
         </is>
       </c>
       <c r="O47" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P47" s="5" t="inlineStr">
@@ -6726,12 +6726,12 @@
       </c>
       <c r="N48" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ nakaz EPU może uruchamiać termin na reakcję, a czas może być krótki albo dane mogą wymagać szybkiego potwierdzenia. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce stwarza bezpośrednie ryzyko dla członka zarządu — jeśli spółka nie złoży sprzeciwu w EPU w terminie, nakaz się uprawomocni. Wierzyciel uruchomi egzekucję, a po jej bezskuteczności skieruje roszczenie bezpośrednio do Ciebie z art. 299 KSH. W EPU termin na sprzeciw jest ściśle liczony od doręczenia — pilność wynika z krótkiego czasu i wymogów elektronicznego postępowania.</t>
         </is>
       </c>
       <c r="O48" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P48" s="5" t="inlineStr">
@@ -6833,12 +6833,12 @@
       </c>
       <c r="N49" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji. Nakaz przeciwko spółce nie zawsze jest dokumentem bezpośrednio skierowanym do członka zarządu, ale może być ważny dla oceny ryzyka odpowiedzialności członka zarządu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce może w konsekwencji prowadzić do osobistej odpowiedzialności członka zarządu z art. 299 KSH — jeśli egzekucja przeciwko spółce okaże się bezskuteczna. Masz jeszcze czas na weryfikację, ale termin na sprzeciw spółki w EPU jest ściśle określony i liczony od doręczenia.</t>
         </is>
       </c>
       <c r="O49" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P49" s="5" t="inlineStr">
@@ -6940,12 +6940,12 @@
       </c>
       <c r="N50" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji. Nakaz EPU przeciwko spółce może być istotny jako dokument pokazujący etap sprawy, ale sam w sobie nie musi jeszcze oznaczać dokumentu bezpośrednio skierowanego do członka zarządu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU przeciwko spółce wymaga sprawdzenia, czy spółka podjęła już działania. W EPU brak sprzeciwu w terminie powoduje uprawomocnienie nakazu i może w przyszłości przełożyć się na ryzyko z art. 299 KSH dla członka zarządu.</t>
         </is>
       </c>
       <c r="O50" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P50" s="5" t="inlineStr">
@@ -7047,12 +7047,12 @@
       </c>
       <c r="N51" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ nakaz EPU może uruchamiać termin na reakcję, a czas może być krótki albo dane mogą wymagać szybkiego potwierdzenia. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce stwarza bezpośrednie ryzyko dla członka zarządu — jeśli spółka nie złoży sprzeciwu w EPU w terminie, nakaz się uprawomocni. Wierzyciel uruchomi egzekucję, a po jej bezskuteczności skieruje roszczenie bezpośrednio do Ciebie z art. 299 KSH. W EPU termin na sprzeciw jest ściśle liczony od doręczenia — pilność wynika z krótkiego czasu i wymogów elektronicznego postępowania.</t>
         </is>
       </c>
       <c r="O51" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata nakazu, treść pouczenia oraz to, czy dokument dotyczy wyłącznie spółki, czy może mieć znaczenie dla sytuacji obecnego albo byłego członka zarządu.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Dodaj 'byłego' w tekstach EPU_NAKAZ_SPOLKA (art. 299 KSH)
'członka zarządu' -> 'byłego członka zarządu' w user_risk_explanation_base
i user_practical_meaning_base dla 13 scenariuszy EPU_NAKAZ_SPOLKA.
Filtr _K4_BYLEGO_RE w _clean() automatycznie przywróci 'członka zarządu'
gdy K4=BOARD_ACTIVE.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -5768,7 +5768,7 @@
       </c>
       <c r="O39" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P39" s="5" t="inlineStr">
@@ -5870,12 +5870,12 @@
       </c>
       <c r="N40" s="5" t="inlineStr">
         <is>
-          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce może w konsekwencji prowadzić do osobistej odpowiedzialności członka zarządu z art. 299 KSH — jeśli egzekucja przeciwko spółce okaże się bezskuteczna. Masz jeszcze czas na weryfikację, ale termin na sprzeciw spółki w EPU jest ściśle określony i liczony od doręczenia.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce może w konsekwencji prowadzić do osobistej odpowiedzialności byłego członka zarządu z art. 299 KSH — jeśli egzekucja przeciwko spółce okaże się bezskuteczna. Masz jeszcze czas na weryfikację, ale termin na sprzeciw spółki w EPU jest ściśle określony i liczony od doręczenia.</t>
         </is>
       </c>
       <c r="O40" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P40" s="5" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="O41" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P41" s="5" t="inlineStr">
@@ -6084,12 +6084,12 @@
       </c>
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce może w konsekwencji prowadzić do osobistej odpowiedzialności członka zarządu z art. 299 KSH — jeśli egzekucja przeciwko spółce okaże się bezskuteczna. Masz jeszcze czas na weryfikację, ale termin na sprzeciw spółki w EPU jest ściśle określony i liczony od doręczenia.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce może w konsekwencji prowadzić do osobistej odpowiedzialności byłego członka zarządu z art. 299 KSH — jeśli egzekucja przeciwko spółce okaże się bezskuteczna. Masz jeszcze czas na weryfikację, ale termin na sprzeciw spółki w EPU jest ściśle określony i liczony od doręczenia.</t>
         </is>
       </c>
       <c r="O42" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P42" s="5" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="O43" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P43" s="5" t="inlineStr">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="O44" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P44" s="5" t="inlineStr">
@@ -6405,12 +6405,12 @@
       </c>
       <c r="N45" s="5" t="inlineStr">
         <is>
-          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce może w konsekwencji prowadzić do osobistej odpowiedzialności członka zarządu z art. 299 KSH — jeśli egzekucja przeciwko spółce okaże się bezskuteczna. Masz jeszcze czas na weryfikację, ale termin na sprzeciw spółki w EPU jest ściśle określony i liczony od doręczenia.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce może w konsekwencji prowadzić do osobistej odpowiedzialności byłego członka zarządu z art. 299 KSH — jeśli egzekucja przeciwko spółce okaże się bezskuteczna. Masz jeszcze czas na weryfikację, ale termin na sprzeciw spółki w EPU jest ściśle określony i liczony od doręczenia.</t>
         </is>
       </c>
       <c r="O45" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P45" s="5" t="inlineStr">
@@ -6517,7 +6517,7 @@
       </c>
       <c r="O46" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P46" s="5" t="inlineStr">
@@ -6624,7 +6624,7 @@
       </c>
       <c r="O47" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P47" s="5" t="inlineStr">
@@ -6731,7 +6731,7 @@
       </c>
       <c r="O48" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P48" s="5" t="inlineStr">
@@ -6833,12 +6833,12 @@
       </c>
       <c r="N49" s="5" t="inlineStr">
         <is>
-          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce może w konsekwencji prowadzić do osobistej odpowiedzialności członka zarządu z art. 299 KSH — jeśli egzekucja przeciwko spółce okaże się bezskuteczna. Masz jeszcze czas na weryfikację, ale termin na sprzeciw spółki w EPU jest ściśle określony i liczony od doręczenia.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) wydany przeciwko spółce może w konsekwencji prowadzić do osobistej odpowiedzialności byłego członka zarządu z art. 299 KSH — jeśli egzekucja przeciwko spółce okaże się bezskuteczna. Masz jeszcze czas na weryfikację, ale termin na sprzeciw spółki w EPU jest ściśle określony i liczony od doręczenia.</t>
         </is>
       </c>
       <c r="O49" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P49" s="5" t="inlineStr">
@@ -6945,7 +6945,7 @@
       </c>
       <c r="O50" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P50" s="5" t="inlineStr">
@@ -7052,7 +7052,7 @@
       </c>
       <c r="O51" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany do spółki — właściwą reakcją spółki jest sprzeciw złożony w postępowaniu elektronicznym w terminie wynikającym z doręczenia i pouczenia. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej i rozpatrywana jest w trybie zwykłym. Brak sprzeciwu spowoduje uprawomocnienie nakazu i otworzy wierzycielowi drogę do egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje złożyć sprzeciw w EPU.</t>
         </is>
       </c>
       <c r="P51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Dodaj 'byłego' w tekstach EPU_NAKAZ_CZLONEK_ZARZADU (pominięcie z poprzedniego commitu)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -4526,12 +4526,12 @@
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P28" s="5" t="inlineStr">
@@ -4641,12 +4641,12 @@
       </c>
       <c r="N29" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie jako członka zarządu. Masz jeszcze czas na złożenie sprzeciwu w EPU, ale wymaga to weryfikacji: daty doręczenia, treści pouczenia oraz podstawy roszczenia. W EPU sprzeciw może być początkowo uproszczony — ważne jest złożenie go w terminie.</t>
+          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu. Masz jeszcze czas na złożenie sprzeciwu w EPU, ale wymaga to weryfikacji: daty doręczenia, treści pouczenia oraz podstawy roszczenia. W EPU sprzeciw może być początkowo uproszczony — ważne jest złożenie go w terminie.</t>
         </is>
       </c>
       <c r="O29" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P29" s="5" t="inlineStr">
@@ -4756,12 +4756,12 @@
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
         </is>
       </c>
       <c r="O30" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P30" s="5" t="inlineStr">
@@ -4867,12 +4867,12 @@
       </c>
       <c r="N31" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie jako członka zarządu. Masz jeszcze czas na złożenie sprzeciwu w EPU, ale wymaga to weryfikacji: daty doręczenia, treści pouczenia oraz podstawy roszczenia. W EPU sprzeciw może być początkowo uproszczony — ważne jest złożenie go w terminie.</t>
+          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu. Masz jeszcze czas na złożenie sprzeciwu w EPU, ale wymaga to weryfikacji: daty doręczenia, treści pouczenia oraz podstawy roszczenia. W EPU sprzeciw może być początkowo uproszczony — ważne jest złożenie go w terminie.</t>
         </is>
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P31" s="5" t="inlineStr">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P32" s="5" t="inlineStr">
@@ -5089,12 +5089,12 @@
       </c>
       <c r="N33" s="5" t="inlineStr">
         <is>
-          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
         </is>
       </c>
       <c r="O33" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P33" s="5" t="inlineStr">
@@ -5200,12 +5200,12 @@
       </c>
       <c r="N34" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie jako członka zarządu. Masz jeszcze czas na złożenie sprzeciwu w EPU, ale wymaga to weryfikacji: daty doręczenia, treści pouczenia oraz podstawy roszczenia. W EPU sprzeciw może być początkowo uproszczony — ważne jest złożenie go w terminie.</t>
+          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu. Masz jeszcze czas na złożenie sprzeciwu w EPU, ale wymaga to weryfikacji: daty doręczenia, treści pouczenia oraz podstawy roszczenia. W EPU sprzeciw może być początkowo uproszczony — ważne jest złożenie go w terminie.</t>
         </is>
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P34" s="5" t="inlineStr">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr">
@@ -5422,12 +5422,12 @@
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
         </is>
       </c>
       <c r="O36" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P36" s="5" t="inlineStr">
@@ -5537,12 +5537,12 @@
       </c>
       <c r="N37" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie jako członka zarządu. Masz jeszcze czas na złożenie sprzeciwu w EPU, ale wymaga to weryfikacji: daty doręczenia, treści pouczenia oraz podstawy roszczenia. W EPU sprzeciw może być początkowo uproszczony — ważne jest złożenie go w terminie.</t>
+          <t>Nakaz z EPU jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu. Masz jeszcze czas na złożenie sprzeciwu w EPU, ale wymaga to weryfikacji: daty doręczenia, treści pouczenia oraz podstawy roszczenia. W EPU sprzeciw może być początkowo uproszczony — ważne jest złożenie go w terminie.</t>
         </is>
       </c>
       <c r="O37" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P37" s="5" t="inlineStr">
@@ -5652,12 +5652,12 @@
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
+          <t>Nakaz zapłaty z EPU (e-Sądu) skierowany bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że wierzyciel dochodzi już Twojej odpowiedzialności osobistej. Termin na sprzeciw w EPU jest ściśle określony od doręczenia i nie podlega przedłużeniu — jego upływ bez reakcji spowoduje uprawomocnienie nakazu.</t>
         </is>
       </c>
       <c r="O38" s="5" t="inlineStr">
         <is>
-          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
+          <t>Nakaz z EPU (e-Sądu) jest skierowany bezpośrednio do Ciebie jako byłego członka zarządu — wierzyciel dochodzi Twojej odpowiedzialności osobistej. Właściwą reakcją jest sprzeciw złożony w postępowaniu elektronicznym w terminie wskazanym w pouczeniu. W EPU sprzeciw może być uproszczony — nie musi od razu zawierać wszystkich zarzutów, ale musi być złożony w terminie. Po skutecznym sprzeciwie sprawa automatycznie trafia do sądu właściwości ogólnej. Kluczowe do ustalenia: data doręczenia, treść pouczenia i termin na sprzeciw.</t>
         </is>
       </c>
       <c r="P38" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Popraw opisy oceny ryzyka dla wezwań sądowych (32 scenariusze)
- WEZWANIE_SADOWE_CZLONEK_ZARZADU (15 szt.): konkretny opis wezwania
  sądowego, konsekwencje braku reakcji (wyrok zaoczny), 'byłego członka
  zarządu' auto-filtrowane przez _K4_BYLEGO_RE dla BOARD_ACTIVE
- WEZWANIE_SADOWE_SPOLKA (17 szt.): mechanizm art. 299 KSH, wyrok zaoczny
  jako ryzyko, zdanie o pełnomocniku auto-zastępowane dla BOARD_ACTIVE
- Teksty różnicowane wg risk_level (URGENT/HIGH/MEDIUM/LOW)
- CSV i Excel zsynchronizowane

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -16856,12 +16856,12 @@
       </c>
       <c r="N142" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że sąd wymaga Twojej odpowiedzi lub stawiennictwa. Masz jeszcze czas na weryfikację, ale termin i zakres wymaganej reakcji muszą zostać ustalone natychmiast.</t>
         </is>
       </c>
       <c r="O142" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P142" s="5" t="inlineStr">
@@ -16963,12 +16963,12 @@
       </c>
       <c r="N143" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że postępowanie jest już w toku i sąd wymaga Twojego działania w ściśle określonym terminie. Brak reakcji może skutkować wyrokiem zaocznym lub utratą możliwości obrony.</t>
         </is>
       </c>
       <c r="O143" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P143" s="5" t="inlineStr">
@@ -17070,12 +17070,12 @@
       </c>
       <c r="N144" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że sąd wymaga Twojej odpowiedzi lub stawiennictwa. Masz jeszcze czas na weryfikację, ale termin i zakres wymaganej reakcji muszą zostać ustalone natychmiast.</t>
         </is>
       </c>
       <c r="O144" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P144" s="5" t="inlineStr">
@@ -17177,12 +17177,12 @@
       </c>
       <c r="N145" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane do Ciebie jako byłego członka zarządu wymaga sprawdzenia treści i terminu. Ryzyko jest umiarkowane, ale brak weryfikacji może spowodować utratę możliwości procesowego działania.</t>
         </is>
       </c>
       <c r="O145" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P145" s="5" t="inlineStr">
@@ -17284,12 +17284,12 @@
       </c>
       <c r="N146" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że postępowanie jest już w toku i sąd wymaga Twojego działania w ściśle określonym terminie. Brak reakcji może skutkować wyrokiem zaocznym lub utratą możliwości obrony.</t>
         </is>
       </c>
       <c r="O146" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P146" s="5" t="inlineStr">
@@ -17391,12 +17391,12 @@
       </c>
       <c r="N147" s="5" t="inlineStr">
         <is>
-          <t>Wysokie ryzyko wynika z połączenia rodzaju dokumentu, potrzeby weryfikacji terminu oraz niepewności danych wymagających sprawdzenia. To najskuteczniejsza ścieżka realnej obrony — pismo przygotowawcze musi zawierać konkretne zarzuty i dowody, nie ogólne zaprzeczenia.</t>
+          <t>Wezwanie sądowe skierowane bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że sąd wymaga Twojej odpowiedzi lub stawiennictwa. Masz jeszcze czas na weryfikację, ale termin i zakres wymaganej reakcji muszą zostać ustalone natychmiast.</t>
         </is>
       </c>
       <c r="O147" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P147" s="5" t="inlineStr">
@@ -17502,12 +17502,12 @@
       </c>
       <c r="N148" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane do Ciebie jako byłego członka zarządu wymaga sprawdzenia treści i terminu. Ryzyko jest umiarkowane, ale brak weryfikacji może spowodować utratę możliwości procesowego działania.</t>
         </is>
       </c>
       <c r="O148" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P148" s="5" t="inlineStr">
@@ -17609,12 +17609,12 @@
       </c>
       <c r="N149" s="5" t="inlineStr">
         <is>
-          <t>Podwyższona pilność wynika przede wszystkim z rodzaju dokumentu oraz możliwego biegu terminu na reakcję. Brak pełnych dokumentów ogranicza pewność wstępnej oceny. Na tym etapie ocena ma charakter wstępny, bo nie widzę treści pisma przygotowawczego strony powodowej.</t>
+          <t>Wezwanie sądowe skierowane bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że postępowanie jest już w toku i sąd wymaga Twojego działania w ściśle określonym terminie. Brak reakcji może skutkować wyrokiem zaocznym lub utratą możliwości obrony.</t>
         </is>
       </c>
       <c r="O149" s="5" t="inlineStr">
         <is>
-          <t>W praktyce najpierw trzeba potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P149" s="5" t="inlineStr">
@@ -17720,12 +17720,12 @@
       </c>
       <c r="N150" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że sąd wymaga Twojej odpowiedzi lub stawiennictwa. Masz jeszcze czas na weryfikację, ale termin i zakres wymaganej reakcji muszą zostać ustalone natychmiast.</t>
         </is>
       </c>
       <c r="O150" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P150" s="5" t="inlineStr">
@@ -17827,12 +17827,12 @@
       </c>
       <c r="N151" s="5" t="inlineStr">
         <is>
-          <t>Sprawa ma niższy poziom pilności, ale nadal warto sprawdzić podstawowe dane i dokumenty. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane do Ciebie jako byłego członka zarządu jest na tym etapie oceniane jako niższe ryzyko. Warto jednak potwierdzić treść wezwania i termin, aby nie przeoczyć wymaganych działań.</t>
         </is>
       </c>
       <c r="O151" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P151" s="5" t="inlineStr">
@@ -17934,12 +17934,12 @@
       </c>
       <c r="N152" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane do Ciebie jako byłego członka zarządu wymaga sprawdzenia treści i terminu. Ryzyko jest umiarkowane, ale brak weryfikacji może spowodować utratę możliwości procesowego działania.</t>
         </is>
       </c>
       <c r="O152" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P152" s="5" t="inlineStr">
@@ -18041,12 +18041,12 @@
       </c>
       <c r="N153" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że postępowanie jest już w toku i sąd wymaga Twojego działania w ściśle określonym terminie. Brak reakcji może skutkować wyrokiem zaocznym lub utratą możliwości obrony.</t>
         </is>
       </c>
       <c r="O153" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P153" s="5" t="inlineStr">
@@ -18148,12 +18148,12 @@
       </c>
       <c r="N154" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że sąd wymaga Twojej odpowiedzi lub stawiennictwa. Masz jeszcze czas na weryfikację, ale termin i zakres wymaganej reakcji muszą zostać ustalone natychmiast.</t>
         </is>
       </c>
       <c r="O154" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P154" s="5" t="inlineStr">
@@ -18255,12 +18255,12 @@
       </c>
       <c r="N155" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane do Ciebie jako byłego członka zarządu wymaga sprawdzenia treści i terminu. Ryzyko jest umiarkowane, ale brak weryfikacji może spowodować utratę możliwości procesowego działania.</t>
         </is>
       </c>
       <c r="O155" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P155" s="5" t="inlineStr">
@@ -18362,12 +18362,12 @@
       </c>
       <c r="N156" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe skierowane bezpośrednio do Ciebie jako byłego członka zarządu oznacza, że postępowanie jest już w toku i sąd wymaga Twojego działania w ściśle określonym terminie. Brak reakcji może skutkować wyrokiem zaocznym lub utratą możliwości obrony.</t>
         </is>
       </c>
       <c r="O156" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane bezpośrednio do Ciebie jako byłego członka zarządu. Kluczowe jest ustalenie czego dokładnie sąd wymaga: stawiennictwa na rozprawie, złożenia pisma procesowego, dostarczenia dokumentów czy złożenia wyjaśnień. Termin wskazany w wezwaniu jest ściśle określony przez sąd i nie podlega automatycznemu przedłużeniu — brak reakcji może skutkować wyrokiem zaocznym lub ograniczeniem możliwości obrony.</t>
         </is>
       </c>
       <c r="P156" s="5" t="inlineStr">
@@ -18469,12 +18469,12 @@
       </c>
       <c r="N157" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki jest istotne z Twojej perspektywy jako byłego członka zarządu — jeśli spółka przegra sprawę lub nie zareaguje, wierzyciel może dochodzić roszczeń bezpośrednio od Ciebie z art. 299 KSH. Masz jeszcze czas na weryfikację, ale działanie jest potrzebne.</t>
         </is>
       </c>
       <c r="O157" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P157" s="5" t="inlineStr">
@@ -18576,12 +18576,12 @@
       </c>
       <c r="N158" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki wymaga sprawdzenia, czy spółka podjęła już działania. Brak reakcji spółki może w przyszłości przełożyć się na ryzyko z art. 299 KSH dla byłego członka zarządu.</t>
         </is>
       </c>
       <c r="O158" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P158" s="5" t="inlineStr">
@@ -18683,12 +18683,12 @@
       </c>
       <c r="N159" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki wymaga pilnej reakcji — jeśli spółka nie odpowie w terminie, sąd może wydać wyrok zaoczny. Po bezskutecznej egzekucji wobec spółki wierzyciel może skierować roszczenie bezpośrednio do Ciebie jako byłego członka zarządu z art. 299 KSH.</t>
         </is>
       </c>
       <c r="O159" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P159" s="5" t="inlineStr">
@@ -18790,12 +18790,12 @@
       </c>
       <c r="N160" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki jest istotne z Twojej perspektywy jako byłego członka zarządu — jeśli spółka przegra sprawę lub nie zareaguje, wierzyciel może dochodzić roszczeń bezpośrednio od Ciebie z art. 299 KSH. Masz jeszcze czas na weryfikację, ale działanie jest potrzebne.</t>
         </is>
       </c>
       <c r="O160" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P160" s="5" t="inlineStr">
@@ -18897,12 +18897,12 @@
       </c>
       <c r="N161" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki wymaga sprawdzenia, czy spółka podjęła już działania. Brak reakcji spółki może w przyszłości przełożyć się na ryzyko z art. 299 KSH dla byłego członka zarządu.</t>
         </is>
       </c>
       <c r="O161" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P161" s="5" t="inlineStr">
@@ -19004,12 +19004,12 @@
       </c>
       <c r="N162" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki wymaga pilnej reakcji — jeśli spółka nie odpowie w terminie, sąd może wydać wyrok zaoczny. Po bezskutecznej egzekucji wobec spółki wierzyciel może skierować roszczenie bezpośrednio do Ciebie jako byłego członka zarządu z art. 299 KSH.</t>
         </is>
       </c>
       <c r="O162" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P162" s="5" t="inlineStr">
@@ -19111,12 +19111,12 @@
       </c>
       <c r="N163" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki jest istotne z Twojej perspektywy jako byłego członka zarządu — jeśli spółka przegra sprawę lub nie zareaguje, wierzyciel może dochodzić roszczeń bezpośrednio od Ciebie z art. 299 KSH. Masz jeszcze czas na weryfikację, ale działanie jest potrzebne.</t>
         </is>
       </c>
       <c r="O163" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P163" s="5" t="inlineStr">
@@ -19218,12 +19218,12 @@
       </c>
       <c r="N164" s="5" t="inlineStr">
         <is>
-          <t>Sprawa ma niższy poziom pilności, ale nadal warto sprawdzić podstawowe dane i dokumenty. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki jest na tym etapie oceniane jako niższe ryzyko bezpośrednie. Warto jednak sprawdzić, czy spółka jest aktywnie reprezentowana w postępowaniu — brak reakcji mógłby doprowadzić do wyroku zaocznego.</t>
         </is>
       </c>
       <c r="O164" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P164" s="5" t="inlineStr">
@@ -19325,12 +19325,12 @@
       </c>
       <c r="N165" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki wymaga sprawdzenia, czy spółka podjęła już działania. Brak reakcji spółki może w przyszłości przełożyć się na ryzyko z art. 299 KSH dla byłego członka zarządu.</t>
         </is>
       </c>
       <c r="O165" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P165" s="5" t="inlineStr">
@@ -19432,12 +19432,12 @@
       </c>
       <c r="N166" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki wymaga pilnej reakcji — jeśli spółka nie odpowie w terminie, sąd może wydać wyrok zaoczny. Po bezskutecznej egzekucji wobec spółki wierzyciel może skierować roszczenie bezpośrednio do Ciebie jako byłego członka zarządu z art. 299 KSH.</t>
         </is>
       </c>
       <c r="O166" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P166" s="5" t="inlineStr">
@@ -19539,12 +19539,12 @@
       </c>
       <c r="N167" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki jest istotne z Twojej perspektywy jako byłego członka zarządu — jeśli spółka przegra sprawę lub nie zareaguje, wierzyciel może dochodzić roszczeń bezpośrednio od Ciebie z art. 299 KSH. Masz jeszcze czas na weryfikację, ale działanie jest potrzebne.</t>
         </is>
       </c>
       <c r="O167" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P167" s="5" t="inlineStr">
@@ -19646,12 +19646,12 @@
       </c>
       <c r="N168" s="5" t="inlineStr">
         <is>
-          <t>Sprawa ma niższy poziom pilności, ale nadal warto sprawdzić podstawowe dane i dokumenty. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki jest na tym etapie oceniane jako niższe ryzyko bezpośrednie. Warto jednak sprawdzić, czy spółka jest aktywnie reprezentowana w postępowaniu — brak reakcji mógłby doprowadzić do wyroku zaocznego.</t>
         </is>
       </c>
       <c r="O168" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P168" s="5" t="inlineStr">
@@ -19753,12 +19753,12 @@
       </c>
       <c r="N169" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki wymaga sprawdzenia, czy spółka podjęła już działania. Brak reakcji spółki może w przyszłości przełożyć się na ryzyko z art. 299 KSH dla byłego członka zarządu.</t>
         </is>
       </c>
       <c r="O169" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P169" s="5" t="inlineStr">
@@ -19860,12 +19860,12 @@
       </c>
       <c r="N170" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki wymaga pilnej reakcji — jeśli spółka nie odpowie w terminie, sąd może wydać wyrok zaoczny. Po bezskutecznej egzekucji wobec spółki wierzyciel może skierować roszczenie bezpośrednio do Ciebie jako byłego członka zarządu z art. 299 KSH.</t>
         </is>
       </c>
       <c r="O170" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P170" s="5" t="inlineStr">
@@ -19967,12 +19967,12 @@
       </c>
       <c r="N171" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki jest istotne z Twojej perspektywy jako byłego członka zarządu — jeśli spółka przegra sprawę lub nie zareaguje, wierzyciel może dochodzić roszczeń bezpośrednio od Ciebie z art. 299 KSH. Masz jeszcze czas na weryfikację, ale działanie jest potrzebne.</t>
         </is>
       </c>
       <c r="O171" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P171" s="5" t="inlineStr">
@@ -20074,12 +20074,12 @@
       </c>
       <c r="N172" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki wymaga sprawdzenia, czy spółka podjęła już działania. Brak reakcji spółki może w przyszłości przełożyć się na ryzyko z art. 299 KSH dla byłego członka zarządu.</t>
         </is>
       </c>
       <c r="O172" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P172" s="5" t="inlineStr">
@@ -20181,12 +20181,12 @@
       </c>
       <c r="N173" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Wezwanie sądowe dotyczące spółki wymaga pilnej reakcji — jeśli spółka nie odpowie w terminie, sąd może wydać wyrok zaoczny. Po bezskutecznej egzekucji wobec spółki wierzyciel może skierować roszczenie bezpośrednio do Ciebie jako byłego członka zarządu z art. 299 KSH.</t>
         </is>
       </c>
       <c r="O173" s="5" t="inlineStr">
         <is>
-          <t>W praktyce należy potwierdzić datę doręczenia, sposób liczenia terminu, adresata pisma, podstawę roszczenia oraz dokumenty dotyczące pełnienia funkcji w zarządzie i aktualności wpisu w KRS.</t>
+          <t>Wezwanie sądowe jest skierowane do spółki. Właściwa reakcja zależy od treści wezwania: może to być stawiennictwo pełnomocnika spółki na rozprawie, złożenie pisma procesowego lub dostarczenie dokumentów. Brak reakcji spółki może doprowadzić do wyroku zaocznego i egzekucji, a po jej bezskuteczności — do roszczenia bezpośrednio wobec Ciebie jako byłego członka zarządu z art. 299 KSH. Kluczowe jest ustalenie, czy spółka ma pełnomocnika procesowego i czy planuje zareagować na wezwanie.</t>
         </is>
       </c>
       <c r="P173" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Napraw treść oceny ryzyka dla opcji 'Inne / nie wiem'
- Lead paragraph nie mówi już 'Na inne / nie wiem masz X dni' — zamiast tego
  'Rodzaj pisma nie został jednoznacznie ustalony. Szacowany czas na reakcję: N dni.'
- Komunikat identyfikacyjny ('Najpierw ustalić, czy pismo jest pozwem...') jest teraz
  PIERWSZYM key_context zamiast ostatniego fallbacku
- Nowy CTA dla nieznanego dokumentu: Audyt 48h służy ustaleniu rodzaju pisma,
  nie ostrzega przedwcześnie o 'pozwie przeciwko członkowi zarządu'
- Nowy wariant K6 procedural text: właściwego pisma nie można wskazać bez
  identyfikacji dokumentu
- BASE_010–026: zaktualizowane user_risk_explanation_base — usunięto frazy
  'rodzaj dokumentu' (nieznany) i 'informacja o EPU' (nie dotyczy tej ścieżki)
- Synchronizacja Excela z CSV

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -2703,7 +2703,7 @@
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga weryfikacji i uporządkowania danych. Bez ustalenia rodzaju pisma nie można precyzyjnie ocenić charakteru sprawy — czas na reakcję i dane z formularza wskazują, że nie warto zwlekać.</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga ostrożnej weryfikacji. Brak pewności co do rodzaju dokumentu ogranicza precyzję oceny — nie można wykluczyć, że pismo wymaga szybkiej reakcji.</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga pilnej weryfikacji. Czas na reakcję i dane z formularza wskazują na podwyższoną pilność — jednak bez ustalenia rodzaju pisma nie można określić właściwego kierunku działania.</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga weryfikacji i uporządkowania danych. Bez ustalenia rodzaju pisma nie można precyzyjnie ocenić charakteru sprawy — czas na reakcję i dane z formularza wskazują, że nie warto zwlekać.</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga ostrożnej weryfikacji. Brak pewności co do rodzaju dokumentu ogranicza precyzję oceny — nie można wykluczyć, że pismo wymaga szybkiej reakcji.</t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>Podwyższona pilność wynika przede wszystkim z rodzaju dokumentu oraz możliwego biegu terminu na reakcję. Czas na reakcję może być ograniczony, dlatego kluczowe jest potwierdzenie daty doręczenia i treści pouczenia. Dosłanie dokumentów może istotnie zmienić szczegółową ocenę sprawy. Działania równoległe: (1) identyfikacja sygnatury, nadawcy i charakteru żądania, (2) weryfikacja własnego statusu formalnego w KRS i relacji do sprawy, (3) ustalenie czy termin wskazany w piśmie jest terminem procesowym (prekluzja) czy administracyjnym (przywrócalny).</t>
+          <t>Podwyższona pilność wynika z możliwego biegu terminu na reakcję. Czas może być ograniczony — kluczowe jest najpierw ustalenie rodzaju pisma, a następnie potwierdzenie daty doręczenia i treści pouczenia.</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="N17" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga weryfikacji i uporządkowania danych. Bez ustalenia rodzaju pisma nie można precyzyjnie ocenić charakteru sprawy — czas na reakcję i dane z formularza wskazują, że nie warto zwlekać.</t>
         </is>
       </c>
       <c r="O17" s="5" t="inlineStr">
@@ -3452,7 +3452,7 @@
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>Sprawa ma niższy poziom pilności, ale nadal warto sprawdzić podstawowe dane i dokumenty. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa ma niższy poziom pilności, ale brak pewności co do rodzaju dokumentu ogranicza pewność tej oceny. Warto potwierdzić podstawowe dane i ustalić, z jakim pismem masz do czynienia.</t>
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr">
@@ -3559,7 +3559,7 @@
       </c>
       <c r="N19" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga ostrożnej weryfikacji. Brak pewności co do rodzaju dokumentu ogranicza precyzję oceny — nie można wykluczyć, że pismo wymaga szybkiej reakcji.</t>
         </is>
       </c>
       <c r="O19" s="5" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga pilnej weryfikacji. Czas na reakcję i dane z formularza wskazują na podwyższoną pilność — jednak bez ustalenia rodzaju pisma nie można określić właściwego kierunku działania.</t>
         </is>
       </c>
       <c r="O20" s="5" t="inlineStr">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="N21" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga weryfikacji i uporządkowania danych. Bez ustalenia rodzaju pisma nie można precyzyjnie ocenić charakteru sprawy — czas na reakcję i dane z formularza wskazują, że nie warto zwlekać.</t>
         </is>
       </c>
       <c r="O21" s="5" t="inlineStr">
@@ -3880,7 +3880,7 @@
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>Sprawa ma niższy poziom pilności, ale nadal warto sprawdzić podstawowe dane i dokumenty. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa ma niższy poziom pilności, ale brak pewności co do rodzaju dokumentu ogranicza pewność tej oceny. Warto potwierdzić podstawowe dane i ustalić, z jakim pismem masz do czynienia.</t>
         </is>
       </c>
       <c r="O22" s="5" t="inlineStr">
@@ -3987,7 +3987,7 @@
       </c>
       <c r="N23" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga ostrożnej weryfikacji. Brak pewności co do rodzaju dokumentu ogranicza precyzję oceny — nie można wykluczyć, że pismo wymaga szybkiej reakcji.</t>
         </is>
       </c>
       <c r="O23" s="5" t="inlineStr">
@@ -4094,7 +4094,7 @@
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga pilnej weryfikacji. Czas na reakcję i dane z formularza wskazują na podwyższoną pilność — jednak bez ustalenia rodzaju pisma nie można określić właściwego kierunku działania.</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="N25" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga uporządkowania i szybkiej weryfikacji, choć nie musi oznaczać krytycznego terminu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga weryfikacji i uporządkowania danych. Bez ustalenia rodzaju pisma nie można precyzyjnie ocenić charakteru sprawy — czas na reakcję i dane z formularza wskazują, że nie warto zwlekać.</t>
         </is>
       </c>
       <c r="O25" s="5" t="inlineStr">
@@ -4308,7 +4308,7 @@
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga ostrożnej weryfikacji, zwłaszcza jeżeli brakuje danych o doręczeniu, adresacie albo statusie dokumentu. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga ostrożnej weryfikacji. Brak pewności co do rodzaju dokumentu ogranicza precyzję oceny — nie można wykluczyć, że pismo wymaga szybkiej reakcji.</t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr">
@@ -4415,7 +4415,7 @@
       </c>
       <c r="N27" s="5" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji, ponieważ połączenie rodzaju dokumentu, czasu na reakcję albo reguł bezpieczeństwa wskazuje na podwyższoną pilność. Na ocenę wpływają przede wszystkim rodzaj dokumentu, czas na reakcję, informacja o EPU oraz dane wskazane w formularzu.</t>
+          <t>Sprawa wymaga pilnej weryfikacji. Czas na reakcję i dane z formularza wskazują na podwyższoną pilność — jednak bez ustalenia rodzaju pisma nie można określić właściwego kierunku działania.</t>
         </is>
       </c>
       <c r="O27" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Napraw treść oceny ryzyka dla opcji 'Pismo z ZUS / urzędu'
Przyczyna: ORGAN_PUBLICZNY_CZLONEK_ZARZADU miał 0 scenariuszy w CSV 12,
przez co system używał fallbacku DOKUMENT_NIEUSTALONY_PRAWNY z tekstami
o EPU i 'rodzaju dokumentu' — całkowicie nieadekwatnymi dla ZUS.

Zmiany:
- Dodano 13 scenariuszy (BASE_173–BASE_185) dla ORGAN_PUBLICZNY_CZLONEK_ZARZADU
  pokrywających wszystkie kombinacje K2 × risk_level z tekstami ZUS-specyficznymi
- Lead paragraph: skrócony z pełnej etykiety dropdown do 'pismo z ZUS lub
  urzędu skarbowego' (nowa gałąź _ZUS_LEAD_DOC_TYPES w _lead_paragraph())
- Nowe CTA (_CTA_ZUS): 'wymaga wyjaśnień i dokumentów — nie sprzeciwu
  ani odpowiedzi na pozew' zamiast języka sądowego z _CTA_PERSONAL
- Synchronizacja Excela z CSV (185 → 186 wierszy)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -1518,7 +1518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W173"/>
+  <dimension ref="A1:W186"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="8.25" customWidth="1" style="4" min="1" max="1"/>
@@ -20219,6 +20219,1345 @@
       </c>
       <c r="V173" s="5" t="n"/>
       <c r="W173" s="5" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>BASE_173</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Sprawa pilna — pismo organu publicznego ZUS/US, 0-3</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_0_3</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>RISK_URGENT</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Sprawa pilna</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr"/>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — pilna reakcja wymagana.</t>
+        </is>
+      </c>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego dotyczące Twojej odpowiedzialności za zobowiązania spółki wymaga pilnej reakcji. Termin na złożenie wyjaśnień lub odwołania jest ściśle określony w pouczeniu — jego przekroczenie może zamknąć drogę do obrony.</t>
+        </is>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>Ze względu na krótki termin warto jak najszybciej przejść do Audytu 48h, aby ustalić termin, zakres żądania i właściwy tryb odpowiedzi na pismo organu.</t>
+        </is>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S174" t="n">
+        <v>1</v>
+      </c>
+      <c r="T174" t="inlineStr"/>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V174" t="inlineStr"/>
+      <c r="W174" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>BASE_174</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Wysokie ryzyko — pismo organu publicznego ZUS/US, 0-3</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_0_3</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>RISK_HIGH</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Wysokie ryzyko</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr"/>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — szybka weryfikacja i odpowiedź.</t>
+        </is>
+      </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego dotyczące Twojej odpowiedzialności za zobowiązania spółki wymaga przygotowanej odpowiedzi. Właściwą formą jest złożenie wyjaśnień i dokumentów — nie sprzeciw ani pismo do sądu. Czas na reakcję jest ograniczony.</t>
+        </is>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>Warto bez zwłoki przejść do Audytu 48h, aby ocenić treść pisma, termin i możliwe kierunki odpowiedzi — zanim zdecydujesz o dalszych krokach.</t>
+        </is>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S175" t="n">
+        <v>1</v>
+      </c>
+      <c r="T175" t="inlineStr"/>
+      <c r="U175" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V175" t="inlineStr"/>
+      <c r="W175" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>BASE_175</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Sprawa pilna — pismo organu publicznego ZUS/US, 4-7</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_4_7</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>RISK_URGENT</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Sprawa pilna</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr"/>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — pilna reakcja wymagana.</t>
+        </is>
+      </c>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego dotyczące Twojej odpowiedzialności za zobowiązania spółki wymaga pilnej reakcji. Termin na złożenie wyjaśnień lub odwołania jest ściśle określony w pouczeniu — jego przekroczenie może zamknąć drogę do obrony.</t>
+        </is>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>Ze względu na krótki termin warto jak najszybciej przejść do Audytu 48h, aby ustalić termin, zakres żądania i właściwy tryb odpowiedzi na pismo organu.</t>
+        </is>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S176" t="n">
+        <v>1</v>
+      </c>
+      <c r="T176" t="inlineStr"/>
+      <c r="U176" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V176" t="inlineStr"/>
+      <c r="W176" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>BASE_176</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Wysokie ryzyko — pismo organu publicznego ZUS/US, 4-7</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_4_7</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>RISK_HIGH</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Wysokie ryzyko</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr"/>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — szybka weryfikacja i odpowiedź.</t>
+        </is>
+      </c>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego dotyczące Twojej odpowiedzialności za zobowiązania spółki wymaga przygotowanej odpowiedzi. Właściwą formą jest złożenie wyjaśnień i dokumentów — nie sprzeciw ani pismo do sądu. Czas na reakcję jest ograniczony.</t>
+        </is>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>Warto bez zwłoki przejść do Audytu 48h, aby ocenić treść pisma, termin i możliwe kierunki odpowiedzi — zanim zdecydujesz o dalszych krokach.</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S177" t="n">
+        <v>1</v>
+      </c>
+      <c r="T177" t="inlineStr"/>
+      <c r="U177" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V177" t="inlineStr"/>
+      <c r="W177" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>BASE_177</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Średnie ryzyko / braki danych — pismo organu publicznego ZUS/US, 4-7</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_4_7</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>RISK_MEDIUM</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Średnie ryzyko / braki danych</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr"/>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — weryfikacja terminu i zakresu.</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego wymaga weryfikacji i przygotowania właściwej odpowiedzi. Masz jeszcze czas, ale warto bez zwłoki potwierdzić termin określony w pouczeniu i ustalić zakres żądania organu.</t>
+        </is>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>Audyt 48h może pomóc ocenić treść pisma organu, termin i zakres odpowiedzialności — zanim zdecydujesz o formie odpowiedzi.</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S178" t="n">
+        <v>1</v>
+      </c>
+      <c r="T178" t="inlineStr"/>
+      <c r="U178" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V178" t="inlineStr"/>
+      <c r="W178" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>BASE_178</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Wysokie ryzyko — pismo organu publicznego ZUS/US, 8-14</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_8_14</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>RISK_HIGH</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Wysokie ryzyko</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr"/>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — szybka weryfikacja i odpowiedź.</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego dotyczące Twojej odpowiedzialności za zobowiązania spółki wymaga przygotowanej odpowiedzi. Właściwą formą jest złożenie wyjaśnień i dokumentów — nie sprzeciw ani pismo do sądu. Czas na reakcję jest ograniczony.</t>
+        </is>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>Warto bez zwłoki przejść do Audytu 48h, aby ocenić treść pisma, termin i możliwe kierunki odpowiedzi — zanim zdecydujesz o dalszych krokach.</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S179" t="n">
+        <v>1</v>
+      </c>
+      <c r="T179" t="inlineStr"/>
+      <c r="U179" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V179" t="inlineStr"/>
+      <c r="W179" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>BASE_179</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Średnie ryzyko / braki danych — pismo organu publicznego ZUS/US, 8-14</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_8_14</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>RISK_MEDIUM</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Średnie ryzyko / braki danych</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr"/>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — weryfikacja terminu i zakresu.</t>
+        </is>
+      </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego wymaga weryfikacji i przygotowania właściwej odpowiedzi. Masz jeszcze czas, ale warto bez zwłoki potwierdzić termin określony w pouczeniu i ustalić zakres żądania organu.</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>Audyt 48h może pomóc ocenić treść pisma organu, termin i zakres odpowiedzialności — zanim zdecydujesz o formie odpowiedzi.</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S180" t="n">
+        <v>1</v>
+      </c>
+      <c r="T180" t="inlineStr"/>
+      <c r="U180" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V180" t="inlineStr"/>
+      <c r="W180" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>BASE_180</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Niższe ryzyko / prewencja — pismo organu publicznego ZUS/US, 8-14</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_8_14</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>RISK_LOW</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Niższe ryzyko / prewencja</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr"/>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — niższe ryzyko, warto potwierdzić termin.</t>
+        </is>
+      </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego dotyczące Twojej sprawy wskazuje na niższe ryzyko. Właściwa reakcja — wyjaśnienia lub odwołanie — wymaga jednak potwierdzenia terminu, adresata i zakresu żądania.</t>
+        </is>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>Audyt 48h może pomóc ocenić treść pisma organu, termin i zakres odpowiedzialności — zanim zdecydujesz o formie odpowiedzi.</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S181" t="n">
+        <v>1</v>
+      </c>
+      <c r="T181" t="inlineStr"/>
+      <c r="U181" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V181" t="inlineStr"/>
+      <c r="W181" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>BASE_181</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Wysokie ryzyko — pismo organu publicznego ZUS/US, above-14</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_ABOVE_14</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>RISK_HIGH</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Wysokie ryzyko</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr"/>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — szybka weryfikacja i odpowiedź.</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego dotyczące Twojej odpowiedzialności za zobowiązania spółki wymaga przygotowanej odpowiedzi. Właściwą formą jest złożenie wyjaśnień i dokumentów — nie sprzeciw ani pismo do sądu. Czas na reakcję jest ograniczony.</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>Warto bez zwłoki przejść do Audytu 48h, aby ocenić treść pisma, termin i możliwe kierunki odpowiedzi — zanim zdecydujesz o dalszych krokach.</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S182" t="n">
+        <v>1</v>
+      </c>
+      <c r="T182" t="inlineStr"/>
+      <c r="U182" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V182" t="inlineStr"/>
+      <c r="W182" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>BASE_182</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Średnie ryzyko / braki danych — pismo organu publicznego ZUS/US, above-14</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_ABOVE_14</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>RISK_MEDIUM</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Średnie ryzyko / braki danych</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr"/>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — weryfikacja terminu i zakresu.</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego wymaga weryfikacji i przygotowania właściwej odpowiedzi. Masz jeszcze czas, ale warto bez zwłoki potwierdzić termin określony w pouczeniu i ustalić zakres żądania organu.</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>Audyt 48h może pomóc ocenić treść pisma organu, termin i zakres odpowiedzialności — zanim zdecydujesz o formie odpowiedzi.</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S183" t="n">
+        <v>1</v>
+      </c>
+      <c r="T183" t="inlineStr"/>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V183" t="inlineStr"/>
+      <c r="W183" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>BASE_183</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Niższe ryzyko / prewencja — pismo organu publicznego ZUS/US, above-14</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_ABOVE_14</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>RISK_LOW</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Niższe ryzyko / prewencja</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — niższe ryzyko, warto potwierdzić termin.</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego dotyczące Twojej sprawy wskazuje na niższe ryzyko. Właściwa reakcja — wyjaśnienia lub odwołanie — wymaga jednak potwierdzenia terminu, adresata i zakresu żądania.</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>Audyt 48h może pomóc ocenić treść pisma organu, termin i zakres odpowiedzialności — zanim zdecydujesz o formie odpowiedzi.</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S184" t="n">
+        <v>1</v>
+      </c>
+      <c r="T184" t="inlineStr"/>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V184" t="inlineStr"/>
+      <c r="W184" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>BASE_184</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Wysokie ryzyko — pismo organu publicznego ZUS/US, unknown</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>RISK_HIGH</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Wysokie ryzyko</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr"/>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — szybka weryfikacja i odpowiedź.</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego dotyczące Twojej odpowiedzialności za zobowiązania spółki wymaga przygotowanej odpowiedzi. Właściwą formą jest złożenie wyjaśnień i dokumentów — nie sprzeciw ani pismo do sądu. Czas na reakcję jest ograniczony.</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>Warto bez zwłoki przejść do Audytu 48h, aby ocenić treść pisma, termin i możliwe kierunki odpowiedzi — zanim zdecydujesz o dalszych krokach.</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S185" t="n">
+        <v>1</v>
+      </c>
+      <c r="T185" t="inlineStr"/>
+      <c r="U185" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V185" t="inlineStr"/>
+      <c r="W185" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>BASE_185</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Średnie ryzyko / braki danych — pismo organu publicznego ZUS/US, unknown</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>RISK_MEDIUM</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>Średnie ryzyko / braki danych</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu — weryfikacja terminu i zakresu.</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego wymaga weryfikacji i przygotowania właściwej odpowiedzi. Masz jeszcze czas, ale warto bez zwłoki potwierdzić termin określony w pouczeniu i ustalić zakres żądania organu.</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>Audyt 48h może pomóc ocenić treść pisma organu, termin i zakres odpowiedzialności — zanim zdecydujesz o formie odpowiedzi.</t>
+        </is>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S186" t="n">
+        <v>1</v>
+      </c>
+      <c r="T186" t="inlineStr"/>
+      <c r="U186" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="V186" t="inlineStr"/>
+      <c r="W186" t="inlineStr">
         <is>
           <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
         </is>

</xml_diff>

<commit_message>
Napraw 3 błędy wykryte podczas audytu kodu (3 agenty)
- app.py: dodaj K2A do odpowiedzi formularza — K2A_DELIVERY_DATE_UNKNOWN (H=1)
  gdy użytkownik wybiera K2 ręcznie; K2A_DELIVERY_DATE_KNOWN gdy oblicza z daty.
  Brak K2A powodował utratę H=1 z punktacji dla wszystkich ręcznych wyborów K2.
- text_builder.py:328: _clean(next_step_base) uzupełniono o k4_code, by
  korekta frazy 'byłego członka zarządu' działała spójnie we wszystkich polach
- CSV/Excel: dodano BASE_188 (ORGAN_PUBLICZNY + K2_UNKNOWN + RISK_URGENT) —
  kombinacja możliwa po naprawie K2A; bez scenariusza system odpada do
  DOKUMENT_NIEUSTALONY z komunikatem 'bez ustalenia rodzaju pisma'

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -1518,7 +1518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W188"/>
+  <dimension ref="A1:W189"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="8.25" customWidth="1" style="4" min="1" max="1"/>
@@ -21414,6 +21414,106 @@
         </is>
       </c>
       <c r="W188" t="inlineStr">
+        <is>
+          <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>BASE_188</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>AKTYWNY</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>BAZOWY</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Sprawa pilna – pismo organu publicznego ZUS/US, nieznany termin</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>K2_DAYS_LEFT_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>RISK_URGENT</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>Sprawa pilna</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>pismo ZUS lub urzędu skarbowego o odpowiedzialności członka zarządu; wyjaśnienia lub odwołanie, nie sprzeciw; sprawdzić termin z pouczenia, zakres zaległości, okres funkcji</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS / urzędu – wysoki ciężar dokumentu, termin nieznany.</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>Pismo z ZUS lub urzędu skarbowego dotyczące Twojej odpowiedzialności za zobowiązania spółki należy do dokumentów o wysokim ciężarze prawnym. Brak znajomości terminu odpowiedzi dodatkowo zwiększa ryzyko — organ wyznacza termin w pouczeniu, którego przekroczenie może zamknąć drogę do obrony.</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>W praktyce należy potwierdzić: datę doręczenia, termin odpowiedzi wskazany w pouczeniu, zakres zaległości, okres pełnienia funkcji w zarządzie oraz dokumenty potwierdzające brak winy lub wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>W Audycie 48h warto zweryfikować: datę doręczenia, termin odpowiedzi, adresata pisma, zakres zaległości, okres pełnienia funkcji w zarządzie, aktualność wpisu w KRS oraz dokumenty wyłączające odpowiedzialność.</t>
+        </is>
+      </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>W pierwszej kolejności ustal termin odpowiedzi wskazany w pouczeniu pisma — Audyt 48h pozwoli ocenić treść dokumentu, termin i właściwy tryb odpowiedzi.</t>
+        </is>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>To jest automatyczna, orientacyjna ocena ryzyka i pilności sprawy. Nie stanowi porady prawnej, opinii prawnej ani rekomendacji procesowej. Indywidualna rekomendacja ścieżki obrony może zostać przygotowana dopiero po analizie dokumentów w ramach Audytu 48h.</t>
+        </is>
+      </c>
+      <c r="S189" t="n">
+        <v>1</v>
+      </c>
+      <c r="U189" t="inlineStr">
+        <is>
+          <t>ZATWIERDZONA</t>
+        </is>
+      </c>
+      <c r="W189" t="inlineStr">
         <is>
           <t>K3–K6 nie są warunkami wyboru scenariusza bazowego; ich teksty pobieraj z arkusza 6A_Moduly_K3_K6.</t>
         </is>

</xml_diff>

<commit_message>
Sync Excel z CSV (BASE_026 + BASE_188)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -4367,7 +4367,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Sprawa wymaga pilnej weryfikacji. Czas na reakcję i dane z formularza wskazują na podwyższoną pilność — jednak bez ustalenia rodzaju pisma nie można określić właściwego kierunku działania.</t>
+          <t>Sprawa oceniana jest jako pilna ze względu na wysoką niepewność — nie wiadomo jakiego rodzaju jest pismo, a termin na reakcję nie jest znany. Brak kluczowych informacji sam w sobie stanowi ryzyko wymagające szybkiego wyjaśnienia.</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -4382,7 +4382,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Ze względu na pilny charakter sprawy warto przejść do Audytu 48h, aby szybko sprawdzić dokumenty, daty, terminy i możliwe kierunki reakcji.</t>
+          <t>Warto bez zbędnej zwłoki ustalić rodzaj dokumentu i termin reakcji — Audyt 48h umożliwia weryfikację treści pisma, terminów i możliwych kierunków działania.</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">

</xml_diff>

<commit_message>
Uproszczenie formatu pliku testów kontrolnych — czytelniejsze kolumny
Zmieniono 9 długich kolumn na 7 krótkich: nr, priorytet, temat,
dane do kalkulatora, co powinien pokazać wynik, czego NIE wolno w wyniku, uwagi.
Kolumny techniczne (scenariusz bazowy, moduły K3-K6) przeniesione do uwagi.
Zsynchronizowano Excel.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -36189,51 +36189,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>test_id</t>
+          <t>nr</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>obszar</t>
+          <t>priorytet</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>dane testowe</t>
+          <t>temat</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>oczekiwany scenariusz bazowy / zachowanie techniczne</t>
+          <t>dane do kalkulatora</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>oczekiwane moduły K3–K6</t>
+          <t>co powinien pokazać wynik</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>oczekiwany wynik użytkownika</t>
+          <t>czego NIE wolno w wyniku</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>czego NIE wolno pokazać użytkownikowi</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>uwagi</t>
         </is>
@@ -36247,42 +36237,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>ODŁOŻONY – poza MVP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Wiele dokumentów</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Pozew przeciwko spółce + pozew przeciwko członkowi zarządu</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Dokument główny: pozew przeciwko członkowi zarządu</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Zależnie od formularza</t>
+          <t>Wynik mówi, który dokument wymaga reakcji i jakie dokumenty są pomocnicze</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Wynik mówi, który dokument wymaga reakcji i jakie dokumenty są pomocnicze</t>
+          <t>Nazwy reguł wyboru dokumentu</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Nazwy reguł wyboru dokumentu</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>ODŁOŻONY – poza MVP</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Wielodokumentowość nie jest zaimplementowana w app.py (MVP). Odłożyć do kolejnego etapu.</t>
+          <t>Wielodokumentowość nie jest zaimplementowana w app.py (MVP). Odłożyć do kolejnego etapu. | Scenariusz: Dokument główny: pozew przeciwko członkowi zarządu</t>
         </is>
       </c>
     </row>
@@ -36294,42 +36274,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>ODŁOŻONY – poza MVP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Wiele dokumentów</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Nakaz przeciwko spółce + nakaz przeciwko członkowi zarządu</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Dokument główny: nakaz przeciwko członkowi zarządu</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Zależnie od formularza</t>
+          <t>Wynik wskazuje nakaz jako dokument wymagający reakcji</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Wynik wskazuje nakaz jako dokument wymagający reakcji</t>
+          <t>Punktacja wyboru dokumentu</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Punktacja wyboru dokumentu</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>ODŁOŻONY – poza MVP</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Wielodokumentowość nie jest zaimplementowana w app.py (MVP). Odłożyć do kolejnego etapu.</t>
+          <t>Wielodokumentowość nie jest zaimplementowana w app.py (MVP). Odłożyć do kolejnego etapu. | Scenariusz: Dokument główny: nakaz przeciwko członkowi zarządu</t>
         </is>
       </c>
     </row>
@@ -36341,40 +36311,34 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>EPU</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Nakaz EPU + pouczenie + potwierdzenie doręczenia</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Typ EPU zgodny z adresatem; dołącz Blok_EPU</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Zależnie od formularza</t>
+          <t>Wynik wyjaśnia, że sprawa pochodzi z EPU/e-Sądu</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Wynik wyjaśnia, że sprawa pochodzi z EPU/e-Sądu</t>
+          <t>EPU jako kod techniczny bez wyjaśnienia</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>EPU jako kod techniczny bez wyjaśnienia</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>Scenariusz: Typ EPU zgodny z adresatem; dołącz Blok_EPU</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -36384,40 +36348,34 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>Termin konkretny</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Data doręczenia + termin z pouczenia dają 5 dni</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>K2 technicznie może być 4–7 dni</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Dowolne</t>
+          <t>Wynik mówi konkretnie, że zostało ok. 5 dni</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Wynik mówi konkretnie, że zostało ok. 5 dni</t>
+          <t>Ogólnik „około 4–7 dni”, gdy znane jest 5 dni</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Ogólnik „około 4–7 dni”, gdy znane jest 5 dni</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>Scenariusz: K2 technicznie może być 4–7 dni</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -36427,40 +36385,34 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>Twarde reguły</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Krótki termin albo termin niepewny</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Poziom ryzyka może zostać podniesiony</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Dowolne</t>
+          <t>Użytkownik widzi nietechniczne ostrzeżenie o konieczności potwierdzenia terminu</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Użytkownik widzi nietechniczne ostrzeżenie o konieczności potwierdzenia terminu</t>
+          <t>HR01, HR02, HR04 itp.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>HR01, HR02, HR04 itp.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
+          <t>Scenariusz: Poziom ryzyka może zostać podniesiony</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -36470,40 +36422,34 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>Brak dokumentów</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Użytkownik chce tylko wstępną ocenę bez dokumentów</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy po K1/K2/ryzyku</t>
-        </is>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>K3_SUPPORT_BASIC_NO_DOCS</t>
+          <t>Wynik jasno mówi, że ocena jest ograniczona bez dokumentów</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Wynik jasno mówi, że ocena jest ograniczona bez dokumentów</t>
+          <t>Kod K3</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Kod K3</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
+          <t>Scenariusz: Scenariusz bazowy po K1/K2/ryzyku; Moduły: K3_SUPPORT_BASIC_NO_DOCS</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -36513,40 +36459,34 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Dokumenty później</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Użytkownik chce ocenę teraz i dosłanie dokumentów później</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy po K1/K2/ryzyku</t>
-        </is>
-      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>K3_SUPPORT_NOW_DOCS_LATER</t>
+          <t>Wynik wskazuje, jakie dokumenty trzeba później uzupełnić</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Wynik wskazuje, jakie dokumenty trzeba później uzupełnić</t>
+          <t>Kod K3</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Kod K3</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
+          <t>Scenariusz: Scenariusz bazowy po K1/K2/ryzyku; Moduły: K3_SUPPORT_NOW_DOCS_LATER</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -36556,40 +36496,34 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>Gotowość do audytu</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Użytkownik gotowy wysłać dokumenty</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy po K1/K2/ryzyku</t>
-        </is>
-      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>K3_READY_FOR_AUDIT_48H</t>
+          <t>Wynik kieruje do listy dokumentów do Audytu 48h</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Wynik kieruje do listy dokumentów do Audytu 48h</t>
+          <t>Kod K3</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Kod K3</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
+          <t>Scenariusz: Scenariusz bazowy po K1/K2/ryzyku; Moduły: K3_READY_FOR_AUDIT_48H</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -36599,40 +36533,34 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>Status zarządu aktywny</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>K4 = nadal pełnię funkcję</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy nie musi mieć K4</t>
-        </is>
-      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MOD_K4_BOARD_ACTIVE</t>
+          <t>Wynik mówi o potrzebie sprawdzenia aktualnego statusu i adresata pisma</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Wynik mówi o potrzebie sprawdzenia aktualnego statusu i adresata pisma</t>
+          <t>BOARD_ACTIVE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>BOARD_ACTIVE</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+          <t>Scenariusz: Scenariusz bazowy nie musi mieć K4; Moduły: MOD_K4_BOARD_ACTIVE</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -36642,42 +36570,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>KLUCZOWY</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>Status zarządu rezygnacja</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>K4 = rezygnacja/odwołanie</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy nie może nadpisać tego statusem aktywnym</t>
-        </is>
-      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MOD_K4_BOARD_RESIGNED + właściwy K5</t>
+          <t>Wynik mówi o rezygnacji/odwołaniu i dacie skuteczności</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Wynik mówi o rezygnacji/odwołaniu i dacie skuteczności</t>
+          <t>Informacja, że użytkownik nadal pełni funkcję</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Informacja, że użytkownik nadal pełni funkcję</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>KLUCZOWY</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>To test problemu ze SCN_002.</t>
+          <t>To test problemu ze SCN_002. | Scenariusz: Scenariusz bazowy nie może nadpisać tego statusem aktywnym; Moduły: MOD_K4_BOARD_RESIGNED + właściwy K5</t>
         </is>
       </c>
     </row>
@@ -36689,40 +36607,34 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>KLUCZOWY</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>KRS nieznany</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>K4=rezygnacja, K5=nie wiem</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy po K1/K2/ryzyku</t>
-        </is>
-      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MOD_K4_BOARD_RESIGNED + MOD_K5_KRS_UNKNOWN</t>
+          <t>Wynik zaleca sprawdzenie dokumentu rezygnacji/odwołania i aktualnego odpisu KRS</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Wynik zaleca sprawdzenie dokumentu rezygnacji/odwołania i aktualnego odpisu KRS</t>
+          <t>K5_KRS_UNKNOWN</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>K5_KRS_UNKNOWN</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>KLUCZOWY</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
+          <t>Scenariusz: Scenariusz bazowy po K1/K2/ryzyku; Moduły: MOD_K4_BOARD_RESIGNED + MOD_K5_KRS_UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -36732,42 +36644,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>KLUCZOWY</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>Cel: zyskać czas</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>K6 = zyskać czas na przygotowanie obrony</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy po K1/K2/ryzyku</t>
-        </is>
-      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MOD_K6_GOAL_BUY_TIME</t>
+          <t>Wynik mówi o legalnych środkach procesowych i przygotowaniu obrony, a nie o terminie na reakcję</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Wynik mówi o legalnych środkach procesowych i przygotowaniu obrony, a nie o terminie na reakcję</t>
+          <t>Sugestia nadużycia prawa lub działań instrumentalnych</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Sugestia nadużycia prawa lub działań instrumentalnych</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>KLUCZOWY</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Rozróżnić od realnej oceny obrony.</t>
+          <t>Rozróżnić od realnej oceny obrony. | Scenariusz: Scenariusz bazowy po K1/K2/ryzyku; Moduły: MOD_K6_GOAL_BUY_TIME</t>
         </is>
       </c>
     </row>
@@ -36779,40 +36681,34 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>Cel: ocena podstaw obrony</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>K6 = ocenić realne podstawy obrony</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy po K1/K2/ryzyku</t>
-        </is>
-      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MOD_K6_GOAL_DEFENSE</t>
+          <t>Wynik koncentruje się na dokumentach, podstawie roszczenia, terminach i możliwych zarzutach</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Wynik koncentruje się na dokumentach, podstawie roszczenia, terminach i możliwych zarzutach</t>
+          <t>Kod K6</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Kod K6</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
+          <t>Scenariusz: Scenariusz bazowy po K1/K2/ryzyku; Moduły: MOD_K6_GOAL_DEFENSE</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -36822,42 +36718,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>Cel: pismo procesowe</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>K6 = przygotować odpowiednie pismo procesowe</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy po K1/K2/ryzyku</t>
-        </is>
-      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MOD_K6_GOAL_PROCEDURAL_LETTER</t>
+          <t>Wynik wskazuje, że rodzaj pisma zależy od dokumentu: sprzeciw przy nakazie, odpowiedź przy pozwie</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Wynik wskazuje, że rodzaj pisma zależy od dokumentu: sprzeciw przy nakazie, odpowiedź przy pozwie</t>
+          <t>Kod K6</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Kod K6</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Nowa opcja K6.</t>
+          <t>Nowa opcja K6. | Scenariusz: Scenariusz bazowy po K1/K2/ryzyku; Moduły: MOD_K6_GOAL_PROCEDURAL_LETTER</t>
         </is>
       </c>
     </row>
@@ -36869,40 +36755,34 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>Cel: plan + ocena szans</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>K6 = plan działania i ocena szans</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy po K1/K2/ryzyku</t>
-        </is>
-      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MOD_K6_GOAL_PLAN</t>
+          <t>Wynik wskazuje potrzebę uporządkowania planu działania i oceny szans</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Wynik wskazuje potrzebę uporządkowania planu działania i oceny szans</t>
+          <t>Kod K6</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Kod K6</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
+          <t>Scenariusz: Scenariusz bazowy po K1/K2/ryzyku; Moduły: MOD_K6_GOAL_PLAN</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -36912,40 +36792,34 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>Cel niepewny</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>K6 = nie wiem / uporządkowanie sytuacji</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy po K1/K2/ryzyku</t>
-        </is>
-      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>MOD_K6_GOAL_UNKNOWN</t>
+          <t>Wynik pomaga uporządkować możliwe kierunki działania</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Wynik pomaga uporządkować możliwe kierunki działania</t>
+          <t>Kod K6</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Kod K6</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr"/>
+          <t>Scenariusz: Scenariusz bazowy po K1/K2/ryzyku; Moduły: MOD_K6_GOAL_UNKNOWN</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -36955,40 +36829,34 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>Model bazowy + moduły</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Nakaz przeciwko członkowi zarządu, 8–14 dni</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy dla nakazu i terminu</t>
-        </is>
-      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Z formularza</t>
+          <t>Wynik podkreśla znaczenie terminu i treści pouczenia</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Wynik podkreśla znaczenie terminu i treści pouczenia</t>
+          <t>SCN_xxx w wyniku użytkownika</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>SCN_xxx w wyniku użytkownika</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
+          <t>Scenariusz: Scenariusz bazowy dla nakazu i terminu; Moduły: Z formularza</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -36998,40 +36866,34 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>EPU pilny</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Nakaz EPU przeciwko członkowi zarządu, 0–3 dni</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy EPU + RISK_URGENT</t>
-        </is>
-      </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Z formularza</t>
+          <t>Wynik pilny + blok EPU + ostrzeżenie o terminie</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Wynik pilny + blok EPU + ostrzeżenie o terminie</t>
+          <t>HRxx, RISK_URGENT</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>HRxx, RISK_URGENT</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr"/>
+          <t>Scenariusz: Scenariusz bazowy EPU + RISK_URGENT; Moduły: Z formularza</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -37041,42 +36903,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>Pozew spółka — brak EPU</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>K1=K1_POZEW_SPOLKA — sprawdzić, że checkbox EPU jest wyłączony (szary) i epu=False</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Typ POZEW_SPOLKA (nie EPU_POZEW_SPOLKA) — EPU_COMPATIBLE[K1_POZEW_SPOLKA]=NIE wymusza epu=False</t>
-        </is>
-      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Z formularza</t>
+          <t>Wynik standardowy dla POZEW_SPOLKA; nie myli pozwu z nakazem i spółki z członkiem zarządu</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Wynik standardowy dla POZEW_SPOLKA; nie myli pozwu z nakazem i spółki z członkiem zarządu</t>
+          <t>EPU_POZEW_SPOLKA jako typ; blok EPU w wyniku; wewnętrzny typ EPU</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>EPU_POZEW_SPOLKA jako typ; blok EPU w wyniku; wewnętrzny typ EPU</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>EPU jest niedostępne dla K1_POZEW_SPOLKA — checkbox jest wyłączony przez UI. Scenariusze EPU_POZEW_SPOLKA celowo nieosiągalne.</t>
+          <t>EPU jest niedostępne dla K1_POZEW_SPOLKA — checkbox jest wyłączony przez UI. Scenariusze EPU_POZEW_SPOLKA celowo nieosiągalne. | Scenariusz: Typ POZEW_SPOLKA (nie EPU_POZEW_SPOLKA) — EPU_COMPATIBLE[K1_POZEW_SPOLKA]=NIE wymusza epu=False; Moduły: Z formularza</t>
         </is>
       </c>
     </row>
@@ -37088,40 +36940,34 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>Dokument nieustalony</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Niejasny dokument, termin nieznany</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Scenariusz bazowy dokument nieustalony albo fallback</t>
-        </is>
-      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Z formularza</t>
+          <t>Wynik ostrożny, wskazuje potrzebę identyfikacji dokumentu i terminu</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Wynik ostrożny, wskazuje potrzebę identyfikacji dokumentu i terminu</t>
+          <t>komunikaty techniczne fallback</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>komunikaty techniczne fallback</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
+          <t>Scenariusz: Scenariusz bazowy dokument nieustalony albo fallback; Moduły: Z formularza</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -37131,42 +36977,32 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>KLUCZOWY</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>SCN_002 problem</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>K1=K1_NAKAZ_CZLONEK_ZARZADU, K2=K2_DAYS_LEFT_4_7, K3=K3_SUPPORT_BASIC_NO_DOCS, K4=K4_BOARD_RESIGNED, K5=K5_KRS_UNKNOWN, K6=K6_GOAL_BUY_TIME, K7=K7_AMOUNT_10K_50K, EPU=NIE</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Może wybrać bazę odpowiadającą K1/K2/ryzyku, ale wynik musi wynikać z modułów K4–K6</t>
-        </is>
-      </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>K4 rezygnacja + K5 nie wiem + K6 kupić czas</t>
+          <t>Wynik NIE zawiera informacji, że użytkownik nadal pełni funkcję</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Wynik NIE zawiera informacji, że użytkownik nadal pełni funkcję</t>
+          <t>BOARD_ACTIVE; 'nadal pełni funkcję' przy K4=resigned</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>BOARD_ACTIVE; 'nadal pełni funkcję' przy K4=resigned</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>KLUCZOWY</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Test ze zrzutu użytkownika.</t>
+          <t>Test ze zrzutu użytkownika. | Scenariusz: Może wybrać bazę odpowiadającą K1/K2/ryzyku, ale wynik musi wynikać z modułów K4–K6; Moduły: K4 rezygnacja + K5 nie wiem + K6 kupić czas</t>
         </is>
       </c>
     </row>
@@ -37178,40 +37014,34 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>KLUCZOWY</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
           <t>Prywatność i technika</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Dowolny przypadek</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Panel testowy może pokazać technikę</t>
-        </is>
-      </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Dowolne</t>
+          <t>Wynik użytkownika bez techniki</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Wynik użytkownika bez techniki</t>
+          <t>risk_level_code, HRxx, K3/K4/K5/K6 codes, moduły, dynamicznie</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>risk_level_code, HRxx, K3/K4/K5/K6 codes, moduły, dynamicznie</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>KLUCZOWY</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
+          <t>Scenariusz: Panel testowy może pokazać technikę</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -37221,40 +37051,34 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>KLUCZOWY</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>Pismo ZUS / urząd — krótki termin</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>K1=K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU, K2=K2_DAYS_LEFT_0_3, K3=K3_SUPPORT_BASIC_NO_DOCS, K4=K4_BOARD_ACTIVE, K5=K5_NOT_APPLICABLE, K6=K6_GOAL_DEFENSE, K7=K7_AMOUNT_10K_50K, EPU=NIE</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>BASE_173 (RISK_URGENT)</t>
-        </is>
-      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>K3, K4_BOARD_ACTIVE, zus_note (nie urgency_note)</t>
+          <t>Lead: "Na pismo z ZUS lub urzędu skarbowego masz X dni"; treść mówi o piśmie ZUS; CTA o wyjaśnieniach — nie sprzeciwie</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Lead: "Na pismo z ZUS lub urzędu skarbowego masz X dni"; treść mówi o piśmie ZUS; CTA o wyjaśnieniach — nie sprzeciwie</t>
+          <t>"bez ustalenia rodzaju pisma"; "sprzeciw"; "odpowiedź na pozew"; kody techniczne</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>"bez ustalenia rodzaju pisma"; "sprzeciw"; "odpowiedź na pozew"; kody techniczne</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>KLUCZOWY</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
+          <t>Scenariusz: BASE_173 (RISK_URGENT); Moduły: K3, K4_BOARD_ACTIVE, zus_note (nie urgency_note)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -37264,42 +37088,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>KLUCZOWY</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
           <t>Pismo ZUS — 14 dni, RISK_URGENT przez ciężar dokumentu</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>K1=K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU, K2=K2_DAYS_LEFT_8_14 (use_dates=TAK, znana data), K3=K3_SUPPORT_BASIC_NO_DOCS, K4=K4_BOARD_ACTIVE, K5=K5_NOT_APPLICABLE, K6=K6_GOAL_DEFENSE, K7=K7_AMOUNT_10K_50K, EPU=NIE</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>BASE_186 (RISK_URGENT — C=3+P=1+H=3+W=1=8)</t>
-        </is>
-      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>K3, K4_BOARD_ACTIVE, zus_note</t>
+          <t>"wysoki ciężar prawny — niezależnie od długości terminu"; wynik NIE mówi że czas wskazuje na pilność</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>"wysoki ciężar prawny — niezależnie od długości terminu"; wynik NIE mówi że czas wskazuje na pilność</t>
+          <t>"bez ustalenia rodzaju pisma"; "czas na reakcję wskazuje na podwyższoną pilność"; "sprzeciw"</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>"bez ustalenia rodzaju pisma"; "czas na reakcję wskazuje na podwyższoną pilność"; "sprzeciw"</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>KLUCZOWY</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Weryfikuje poprawność BASE_186 — główny błąd zgłoszony przez użytkownika.</t>
+          <t>Weryfikuje poprawność BASE_186 — główny błąd zgłoszony przez użytkownika. | Scenariusz: BASE_186 (RISK_URGENT — C=3+P=1+H=3+W=1=8); Moduły: K3, K4_BOARD_ACTIVE, zus_note</t>
         </is>
       </c>
     </row>
@@ -37311,40 +37125,34 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
           <t>Pismo ZUS — nieznany termin</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>K1=K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU, K2=K2_DAYS_LEFT_UNKNOWN, K3=K3_SUPPORT_BASIC_NO_DOCS, K4=K4_BOARD_ACTIVE, K5=K5_NOT_APPLICABLE, K6=K6_GOAL_DEFENSE, K7=K7_AMOUNT_10K_50K, EPU=NIE</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>BASE_188 (RISK_URGENT) lub BASE_184 (RISK_HIGH) — zależnie od S z K2A</t>
-        </is>
-      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>K3, K4_BOARD_ACTIVE, zus_note</t>
+          <t>Mówi o piśmie ZUS; zaleca potwierdzenie terminu z pouczenia; NIE zawiera "bez ustalenia rodzaju pisma"</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Mówi o piśmie ZUS; zaleca potwierdzenie terminu z pouczenia; NIE zawiera "bez ustalenia rodzaju pisma"</t>
+          <t>"bez ustalenia rodzaju pisma"; "sprzeciw"; kody techniczne</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>"bez ustalenia rodzaju pisma"; "sprzeciw"; kody techniczne</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
+          <t>Scenariusz: BASE_188 (RISK_URGENT) lub BASE_184 (RISK_HIGH) — zależnie od S z K2A; Moduły: K3, K4_BOARD_ACTIVE, zus_note</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -37354,42 +37162,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>KLUCZOWY</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
           <t>Inne/nie wiem + wiele opcji "nie wiem" — RISK_URGENT</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>K1=K1_INNE_NIE_WIEM, K2=K2_DAYS_LEFT_UNKNOWN, K3=K3_SUPPORT_BASIC_NO_DOCS, K4=K4_BOARD_UNKNOWN, K5=K5_KRS_UNKNOWN, K6=K6_GOAL_UNKNOWN, K7=K7_AMOUNT_UNKNOWN, EPU=NIE</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>BASE_026 (K2_UNKNOWN + RISK_URGENT)</t>
-        </is>
-      </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>K3, K4_BOARD_UNKNOWN, K5_KRS_UNKNOWN, K6_GOAL_UNKNOWN, unknown_doc_note</t>
+          <t>"pilna ze względu na wysoką niepewność"; wynik NIE mówi że czas wskazuje na pilność</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>"pilna ze względu na wysoką niepewność"; wynik NIE mówi że czas wskazuje na pilność</t>
+          <t>"Czas na reakcję wskazuje na podwyższoną pilność"; kody techniczne</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>"Czas na reakcję wskazuje na podwyższoną pilność"; kody techniczne</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>KLUCZOWY</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Weryfikuje poprawność BASE_026 po naprawie tekstu.</t>
+          <t>Weryfikuje poprawność BASE_026 po naprawie tekstu. | Scenariusz: BASE_026 (K2_UNKNOWN + RISK_URGENT); Moduły: K3, K4_BOARD_UNKNOWN, K5_KRS_UNKNOWN, K6_GOAL_UNKNOWN, unknown_doc_note</t>
         </is>
       </c>
     </row>
@@ -37401,42 +37199,32 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>KLUCZOWY</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
           <t>Pismo ZUS — cel: pismo procesowe</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>K1=K1_ORGAN_PUBLICZNY_CZLONEK_ZARZADU, K2=K2_DAYS_LEFT_8_14, K3=K3_SUPPORT_BASIC_NO_DOCS, K4=K4_BOARD_ACTIVE, K5=K5_NOT_APPLICABLE, K6=K6_GOAL_PROCEDURAL_LETTER, K7=K7_AMOUNT_10K_50K, EPU=NIE</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>BASE_186 lub BASE_178</t>
-        </is>
-      </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>K6_GOAL_PROCEDURAL_LETTER (wyjaśnienia, nie sprzeciw)</t>
+          <t>K6 text: "wyjaśnienia i dokumenty potwierdzające stanowisko — nie sprzeciw ani odpowiedź na pozew"</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>K6 text: "wyjaśnienia i dokumenty potwierdzające stanowisko — nie sprzeciw ani odpowiedź na pozew"</t>
+          <t>"sprzeciw"; "odpowiedź na pozew"; kody techniczne</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>"sprzeciw"; "odpowiedź na pozew"; kody techniczne</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>KLUCZOWY</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>Kluczowa reguła komunikacyjna dla ZUS.</t>
+          <t>Kluczowa reguła komunikacyjna dla ZUS. | Scenariusz: BASE_186 lub BASE_178; Moduły: K6_GOAL_PROCEDURAL_LETTER (wyjaśnienia, nie sprzeciw)</t>
         </is>
       </c>
     </row>
@@ -37448,42 +37236,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>DO TESTU</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
           <t>Punktacja K2A — ręczny wybór K2</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>K1=K1_INNE_NIE_WIEM, K2=K2_DAYS_LEFT_UNKNOWN (bez zaznaczenia checkboxa daty), K3=K3_SUPPORT_BASIC_NO_DOCS, K4=K4_BOARD_ACTIVE, K5=K5_NOT_APPLICABLE, K6=K6_GOAL_DEFENSE, K7=K7_AMOUNT_10K_50K</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Panel testowy: answers zawiera K2A=K2A_DELIVERY_DATE_UNKNOWN</t>
-        </is>
-      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Brak widocznego modułu K2A w wyniku</t>
+          <t>Panel testowy pokazuje H wyższe o 1 niż bez K2A; klient nie widzi K2A w tekście wyniku</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Panel testowy pokazuje H wyższe o 1 niż bez K2A; klient nie widzi K2A w tekście wyniku</t>
+          <t>K2A_DELIVERY_DATE_UNKNOWN jako widoczny tekst; kody techniczne</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>K2A_DELIVERY_DATE_UNKNOWN jako widoczny tekst; kody techniczne</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>DO TESTU</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Weryfikacja przez panel testowy — klient widzi tylko wynik S i poziom ryzyka.</t>
+          <t>Weryfikacja przez panel testowy — klient widzi tylko wynik S i poziom ryzyka. | Scenariusz: Panel testowy: answers zawiera K2A=K2A_DELIVERY_DATE_UNKNOWN; Moduły: Brak widocznego modułu K2A w wyniku</t>
         </is>
       </c>
     </row>
@@ -37495,42 +37273,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>KLUCZOWY</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
           <t>Walidacja formularza</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Kalkulator po starcie lub po wyczyszczeniu — kliknij "Oblicz ryzyko →" bez zaznaczenia żadnych opcji</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Brak obliczeń — walidacja blokuje wykonanie</t>
-        </is>
-      </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Brak</t>
+          <t>Pojawia się ostrzeżenie z listą brakujących kroków (np. "Krok 1 — Rodzaj pisma, Krok 3 — Czas na reakcję..."); sekcja "Twoja ocena ryzyka" NIE pojawia się</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Pojawia się ostrzeżenie z listą brakujących kroków (np. "Krok 1 — Rodzaj pisma, Krok 3 — Czas na reakcję..."); sekcja "Twoja ocena ryzyka" NIE pojawia się</t>
+          <t>Wynik ryzyka bez wypełnionego formularza</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Wynik ryzyka bez wypełnionego formularza</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>KLUCZOWY</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Testuje nową funkcję walidacji dodaną w app.py.</t>
+          <t>Testuje nową funkcję walidacji dodaną w app.py. | Scenariusz: Brak obliczeń — walidacja blokuje wykonanie; Moduły: Brak</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dodaj PISMO_PROCESOWE_SADOWE do arkusza Excel 3_Typy_dokumentow
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -37554,7 +37554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="23.5" customWidth="1" style="4" min="1" max="1"/>
@@ -38713,47 +38713,94 @@
       </c>
     </row>
     <row r="26" ht="140.4499969482422" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PISMO_PROCESOWE_SADOWE</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Pismo procesowe w toczącym się postępowaniu sądowym</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>sąd</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>członek zarządu / spółka</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>pismo przygotowawcze; odpowiedź na sprzeciw; w odpowiedzi na sprzeciw; replika; podtrzymuję; wnoszę o oddalenie; postępowanie w toku; sprawa w toku; dalsze pisma</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>pismo przygotowawcze; odpowiedź na sprzeciw; w odpowiedzi na sprzeciw</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>termin wskazany w wezwaniu sądu jeśli dotyczy</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>WARUNKOWO</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Dokument wskazuje na kontynuację sporu sądowego. Bez kompletnej dokumentacji (pozwu, sprzeciwu, wcześniejszych pism) rzetelna ocena jest niemożliwa. Jeżeli jest dokumentem głównym — przekierować do Audytu 48h z pełną dokumentacją.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>ORGAN_PUBLICZNY_CZLONEK_ZARZADU</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Pismo z ZUS / urzędu dotyczące odpowiedzialności członka zarządu</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>organ publiczny</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>członek zarządu</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>ZUS; Zakład Ubezpieczeń Społecznych; urząd skarbowy; naczelnik urzędu skarbowego; odpowiedzialność osoby trzeciej; odpowiedzialność członka zarządu; zaległości składkowe; zaległości podatkowe; Ordynacja podatkowa; ustawa o systemie ubezpieczeń społecznych; wezwanie do wyjaśnień; zawiadomienie o wszczęciu postępowania; decyzja</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>organ publiczny informuje o wszczęciu postępowania albo wzywa członka zarządu do wyjaśnień w sprawie odpowiedzialności za zobowiązania spółki</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>termin wskazany w piśmie organu, często na złożenie wyjaśnień albo dokumentów</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>TAK</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr">
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>Odrębna ścieżka od pozwu/nakazu. Nie generować sprzeciwu ani odpowiedzi na pozew; priorytetem są wyjaśnienia, dowody, okres pełnienia funkcji i przesłanki wyłączające odpowiedzialność.</t>
         </is>

</xml_diff>

<commit_message>
Dodaj zasady pracy: CSV+Excel sync, ostrzezenie o tokenach, aktualizacja docs
- CLAUDE.md: nowa sekcja 'Zasady pracy Claude Code' z regula synchronizacji
  CSV i Excela, zasada biezacej aktualizacji dokumentacji, ostrzezenie o tokenach
- CLAUDE.md: zaktualizowano test documents (dodano Lublin_pozew_pko.pdf)
- Excel: zaktualizowano EPU_POZEW_CZLONEK_ZARZADU (nowe slowa kluczowe i sygnaly)
- Excel: dodano regule R06a dla Pozew w EPU (brakowala przy R06 dla nakazu EPU)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -27748,7 +27748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="6.25" customWidth="1" style="4" min="1" max="1"/>
@@ -27985,39 +27985,41 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>R07</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>R06a</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Typ dokumentu</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Wezwanie sądowe skierowane do członka zarządu</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Bardzo silny kandydat</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Może oznaczać konieczność reakcji lub udziału w postępowaniu</t>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Pozew w elektronicznym postepowaniu upominawczym (EPU) przeciwko czlonkowi zarzadu</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Dokument glowny - wysoki priorytet</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Jezeli sygnatura zawiera Nc-e albo wystepuje Sad Rejonowy Lublin-Zachod, dodaj flage EPU. Pozew jest wczesniejszym etapem niz nakaz - nie musi zawierac formuly nakazowej.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>R08</t>
+          <t>R07</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -28027,7 +28029,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Pismo komornicze skierowane do członka zarządu</t>
+          <t>Wezwanie sądowe skierowane do członka zarządu</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
@@ -28040,14 +28042,14 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Wskazuje na etap egzekucyjny albo ryzyko majątkowe</t>
+          <t>Może oznaczać konieczność reakcji lub udziału w postępowaniu</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>R09</t>
+          <t>R08</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -28057,27 +28059,27 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Pozew przeciwko spółce</t>
+          <t>Pismo komornicze skierowane do członka zarządu</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Dokument główny tylko wtedy, gdy brak dokumentu przeciwko członkowi zarządu</t>
+          <t>Bardzo silny kandydat</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Ważny jako kontekst, ale nie zawsze bezpośrednio dotyczy odpowiedzialności osobistej</t>
+          <t>Wskazuje na etap egzekucyjny albo ryzyko majątkowe</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>R10</t>
+          <t>R09</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -28087,11 +28089,11 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Nakaz zapłaty przeciwko spółce</t>
+          <t>Pozew przeciwko spółce</t>
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
@@ -28100,14 +28102,14 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Może być ważny dla późniejszej odpowiedzialności z art. 299 KSH</t>
+          <t>Ważny jako kontekst, ale nie zawsze bezpośrednio dotyczy odpowiedzialności osobistej</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R10</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -28117,27 +28119,27 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Pismo komornicze dotyczące egzekucji przeciwko spółce</t>
+          <t>Nakaz zapłaty przeciwko spółce</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Ważny dokument kontekstowy, czasem główny</t>
+          <t>Dokument główny tylko wtedy, gdy brak dokumentu przeciwko członkowi zarządu</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Szczególnie ważny, jeżeli wskazuje na bezskuteczność egzekucji</t>
+          <t>Może być ważny dla późniejszej odpowiedzialności z art. 299 KSH</t>
         </is>
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -28147,27 +28149,27 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Postanowienie o umorzeniu egzekucji przeciwko spółce z powodu bezskuteczności</t>
+          <t>Pismo komornicze dotyczące egzekucji przeciwko spółce</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Bardzo ważny dokument kontekstowy</t>
+          <t>Ważny dokument kontekstowy, czasem główny</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Może być kluczowy dla sprawy z art. 299 KSH, ale nie zawsze wymaga natychmiastowej reakcji</t>
+          <t>Szczególnie ważny, jeżeli wskazuje na bezskuteczność egzekucji</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -28177,27 +28179,27 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Przedsądowe wezwanie do zapłaty skierowane do członka zarządu</t>
+          <t>Postanowienie o umorzeniu egzekucji przeciwko spółce z powodu bezskuteczności</t>
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Kandydat na dokument główny</t>
+          <t>Bardzo ważny dokument kontekstowy</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Ważne, ale zwykle mniej pilne niż pozew lub nakaz</t>
+          <t>Może być kluczowy dla sprawy z art. 299 KSH, ale nie zawsze wymaga natychmiastowej reakcji</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>R13</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -28207,27 +28209,27 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Przedsądowe wezwanie do zapłaty skierowane do spółki</t>
+          <t>Przedsądowe wezwanie do zapłaty skierowane do członka zarządu</t>
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Dokument pomocniczy</t>
+          <t>Kandydat na dokument główny</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Nie powinien wygrywać z dokumentem sądowym</t>
+          <t>Ważne, ale zwykle mniej pilne niż pozew lub nakaz</t>
         </is>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>R15</t>
+          <t>R14</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -28237,27 +28239,27 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Decyzja ZUS lub decyzja podatkowa dotycząca odpowiedzialności osoby zarządzającej</t>
+          <t>Przedsądowe wezwanie do zapłaty skierowane do spółki</t>
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Silny kandydat na dokument główny</t>
+          <t>Dokument pomocniczy</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Dotyczy odpowiedzialności osobistej, ale może należeć do ścieżki Audyt 48h, nie tylko art. 299 KSH</t>
+          <t>Nie powinien wygrywać z dokumentem sądowym</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>R15</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -28267,57 +28269,57 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Decyzja ZUS lub US skierowana wyłącznie do spółki</t>
+          <t>Decyzja ZUS lub decyzja podatkowa dotycząca odpowiedzialności osoby zarządzającej</t>
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Dokument pomocniczy albo kandydat drugiego rzędu</t>
+          <t>Silny kandydat na dokument główny</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Ważny kontekst, ale niższy priorytet niż decyzja wobec osoby fizycznej</t>
+          <t>Dotyczy odpowiedzialności osobistej, ale może należeć do ścieżki Audyt 48h, nie tylko art. 299 KSH</t>
         </is>
       </c>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>R17</t>
+          <t>R16</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Termin</t>
+          <t>Typ dokumentu</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Dokument zawiera wyraźny termin reakcji: sprzeciw, zarzuty, odpowiedź, odwołanie, skarga, zażalenie</t>
+          <t>Decyzja ZUS lub US skierowana wyłącznie do spółki</t>
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Silny kandydat na dokument główny</t>
+          <t>Dokument pomocniczy albo kandydat drugiego rzędu</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Termin reakcji bardzo zwiększa priorytet dokumentu</t>
+          <t>Ważny kontekst, ale niższy priorytet niż decyzja wobec osoby fizycznej</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>R18</t>
+          <t>R17</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -28327,27 +28329,27 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Dokument wskazuje termin 0–3 dni pozostałe na reakcję</t>
+          <t>Dokument zawiera wyraźny termin reakcji: sprzeciw, zarzuty, odpowiedź, odwołanie, skarga, zażalenie</t>
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Dokument krytyczny</t>
+          <t>Silny kandydat na dokument główny</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Jeżeli termin jest tak krótki, dokument prawie zawsze powinien być główny</t>
+          <t>Termin reakcji bardzo zwiększa priorytet dokumentu</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>R19</t>
+          <t>R18</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -28357,27 +28359,27 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Dokument wskazuje termin 4–7 dni pozostałe na reakcję</t>
+          <t>Dokument wskazuje termin 0–3 dni pozostałe na reakcję</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Dokument bardzo pilny</t>
+          <t>Dokument krytyczny</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Wysoki priorytet</t>
+          <t>Jeżeli termin jest tak krótki, dokument prawie zawsze powinien być główny</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>R20</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -28387,27 +28389,27 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Dokument wskazuje termin 8–14 dni pozostałe na reakcję</t>
+          <t>Dokument wskazuje termin 4–7 dni pozostałe na reakcję</t>
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Dokument pilny</t>
+          <t>Dokument bardzo pilny</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Średnio-wysoki priorytet</t>
+          <t>Wysoki priorytet</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R20</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -28417,27 +28419,27 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Dokument wskazuje termin powyżej 14 dni</t>
+          <t>Dokument wskazuje termin 8–14 dni pozostałe na reakcję</t>
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Dokument mniej pilny</t>
+          <t>Dokument pilny</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Priorytet zależy od typu dokumentu</t>
+          <t>Średnio-wysoki priorytet</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>R22</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -28447,7 +28449,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Nie udało się ustalić terminu reakcji</t>
+          <t>Dokument wskazuje termin powyżej 14 dni</t>
         </is>
       </c>
       <c r="D24" s="5" t="n">
@@ -28455,49 +28457,49 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Kandydat niepewny</t>
+          <t>Dokument mniej pilny</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>AI powinno oznaczyć brak pewności i wskazać konieczność weryfikacji w Audycie 48h</t>
+          <t>Priorytet zależy od typu dokumentu</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>R23</t>
+          <t>R22</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Etap sprawy</t>
+          <t>Termin</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Dokument pochodzi z sądu</t>
+          <t>Nie udało się ustalić terminu reakcji</t>
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Wysoki priorytet</t>
+          <t>Kandydat niepewny</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Sądowe dokumenty mają wyższy priorytet niż korespondencja prywatna</t>
+          <t>AI powinno oznaczyć brak pewności i wskazać konieczność weryfikacji w Audycie 48h</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>R24</t>
+          <t>R23</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -28507,7 +28509,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Dokument pochodzi od komornika</t>
+          <t>Dokument pochodzi z sądu</t>
         </is>
       </c>
       <c r="D26" s="5" t="n">
@@ -28520,14 +28522,14 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Może wskazywać na etap egzekucji lub bezskuteczność egzekucji</t>
+          <t>Sądowe dokumenty mają wyższy priorytet niż korespondencja prywatna</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>R25</t>
+          <t>R24</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -28537,7 +28539,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Dokument pochodzi od ZUS, US albo innego organu</t>
+          <t>Dokument pochodzi od komornika</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
@@ -28550,14 +28552,14 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Szczególnie gdy dotyczy osoby fizycznej</t>
+          <t>Może wskazywać na etap egzekucji lub bezskuteczność egzekucji</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>R26</t>
+          <t>R25</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -28567,147 +28569,147 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Dokument pochodzi od wierzyciela albo kancelarii wierzyciela</t>
+          <t>Dokument pochodzi od ZUS, US albo innego organu</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Średni priorytet</t>
+          <t>Wysoki priorytet</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Ważne, ale niżej niż sąd/organ/komornik</t>
+          <t>Szczególnie gdy dotyczy osoby fizycznej</t>
         </is>
       </c>
     </row>
     <row r="29" ht="60" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>R27</t>
+          <t>R26</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Art. 299 KSH</t>
+          <t>Etap sprawy</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Dokument zawiera frazy: „art. 299 KSH”, „odpowiedzialność członków zarządu”, „bezskuteczność egzekucji”, „zobowiązania spółki”</t>
+          <t>Dokument pochodzi od wierzyciela albo kancelarii wierzyciela</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Bardzo silny sygnał zgodności z celem kalkulatora</t>
+          <t>Średni priorytet</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>AI powinno podnieść priorytet dokumentu</t>
+          <t>Ważne, ale niżej niż sąd/organ/komornik</t>
         </is>
       </c>
     </row>
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>R28</t>
+          <t>R27</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>EPU</t>
+          <t>Art. 299 KSH</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Dokument zawiera sygnaturę „Nc-e” albo wskazuje Sąd Rejonowy Lublin-Zachód w Lublinie</t>
+          <t>Dokument zawiera frazy: „art. 299 KSH”, „odpowiedzialność członków zarządu”, „bezskuteczność egzekucji”, „zobowiązania spółki”</t>
         </is>
       </c>
       <c r="D30" s="5" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Dodaj flagę EPU</t>
+          <t>Bardzo silny sygnał zgodności z celem kalkulatora</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Nie musi samodzielnie przesądzać wyboru, ale podnosi pilność</t>
+          <t>AI powinno podnieść priorytet dokumentu</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R28</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Data dokumentu</t>
+          <t>EPU</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Dokument jest najnowszy spośród dokumentów o podobnym priorytecie</t>
+          <t>Dokument zawiera sygnaturę „Nc-e” albo wskazuje Sąd Rejonowy Lublin-Zachód w Lublinie</t>
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Reguła pomocnicza</t>
+          <t>Dodaj flagę EPU</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Stosować tylko przy remisie albo bardzo zbliżonym wyniku</t>
+          <t>Nie musi samodzielnie przesądzać wyboru, ale podnosi pilność</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>R30</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Jakość odczytu</t>
+          <t>Data dokumentu</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Dokument został odczytany z wysoką pewnością OCR/tekstu</t>
+          <t>Dokument jest najnowszy spośród dokumentów o podobnym priorytecie</t>
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Podnosi pewność wyboru</t>
+          <t>Reguła pomocnicza</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Nie powinno decydować samo w sobie</t>
+          <t>Stosować tylko przy remisie albo bardzo zbliżonym wyniku</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>R31</t>
+          <t>R30</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -28717,103 +28719,121 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Dokument został odczytany z niską pewnością OCR/tekstu</t>
+          <t>Dokument został odczytany z wysoką pewnością OCR/tekstu</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>-10</v>
+        <v>5</v>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Obniża pewność wyboru</t>
+          <t>Podnosi pewność wyboru</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>AI powinno pokazać ostrzeżenie o konieczności weryfikacji</t>
+          <t>Nie powinno decydować samo w sobie</t>
         </is>
       </c>
     </row>
     <row r="34" ht="60" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>R31</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Dokument pomocniczy</t>
+          <t>Jakość odczytu</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Dokument jest fakturą, umową, odpisem KRS, korespondencją handlową, potwierdzeniem przelewu albo dokumentem księgowym</t>
+          <t>Dokument został odczytany z niską pewnością OCR/tekstu</t>
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>-20</v>
+        <v>-10</v>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Zwykle nie wybierać jako główny</t>
+          <t>Obniża pewność wyboru</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Może być ważny dla Audytu 48h, ale nie jako dokument wymagający reakcji</t>
+          <t>AI powinno pokazać ostrzeżenie o konieczności weryfikacji</t>
         </is>
       </c>
     </row>
     <row r="35" ht="45" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Dokument pomocniczy</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Dokument jest fakturą, umową, odpisem KRS, korespondencją handlową, potwierdzeniem przelewu albo dokumentem księgowym</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>-20</v>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Zwykle nie wybierać jako główny</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Może być ważny dla Audytu 48h, ale nie jako dokument wymagający reakcji</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
           <t>R33</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Dokument obcy tematycznie</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>Dokument nie jest dokumentem prawnym albo nie dotyczy odpowiedzialności zarządu/spółki</t>
         </is>
       </c>
-      <c r="D35" s="5" t="n">
+      <c r="D36" s="5" t="n">
         <v>-100</v>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>Nie wybierać jako dokument główny</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>Pokazać komunikat: „Wczytany dokument wydaje się nie być właściwy dla kalkulatora”</t>
         </is>
       </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="25" t="n"/>
-      <c r="B36" s="26" t="inlineStr">
-        <is>
-          <t>Kolejność oceny powinna być następująca:</t>
-        </is>
-      </c>
-      <c r="C36" s="69" t="n"/>
-      <c r="D36" s="25" t="n"/>
-      <c r="E36" s="25" t="n"/>
-      <c r="F36" s="25" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="25" t="n"/>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>1. Czy dokument dotyczy członka zarządu?</t>
-        </is>
-      </c>
-      <c r="C37" s="37" t="n"/>
+      <c r="B37" s="26" t="inlineStr">
+        <is>
+          <t>Kolejność oceny powinna być następująca:</t>
+        </is>
+      </c>
+      <c r="C37" s="69" t="n"/>
       <c r="D37" s="25" t="n"/>
       <c r="E37" s="25" t="n"/>
       <c r="F37" s="25" t="n"/>
@@ -28822,7 +28842,7 @@
       <c r="A38" s="25" t="n"/>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>2. Czy dokument uruchamia termin na reakcję?</t>
+          <t>1. Czy dokument dotyczy członka zarządu?</t>
         </is>
       </c>
       <c r="C38" s="37" t="n"/>
@@ -28834,7 +28854,7 @@
       <c r="A39" s="25" t="n"/>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>3. Czy dokument dotyczy odpowiedzialności z art. 299 KSH albo podobnego ryzyka osobistego?</t>
+          <t>2. Czy dokument uruchamia termin na reakcję?</t>
         </is>
       </c>
       <c r="C39" s="37" t="n"/>
@@ -28846,7 +28866,7 @@
       <c r="A40" s="25" t="n"/>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>4. Czy dokument pochodzi z sądu, komornika, organu lub wierzyciela?</t>
+          <t>3. Czy dokument dotyczy odpowiedzialności z art. 299 KSH albo podobnego ryzyka osobistego?</t>
         </is>
       </c>
       <c r="C40" s="37" t="n"/>
@@ -28858,7 +28878,7 @@
       <c r="A41" s="25" t="n"/>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>5. Czy dokument jest aktualny i ma biegnący termin?</t>
+          <t>4. Czy dokument pochodzi z sądu, komornika, organu lub wierzyciela?</t>
         </is>
       </c>
       <c r="C41" s="37" t="n"/>
@@ -28870,7 +28890,7 @@
       <c r="A42" s="25" t="n"/>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>6. Dopiero na końcu — jaka jest data dokumentu.</t>
+          <t>5. Czy dokument jest aktualny i ma biegnący termin?</t>
         </is>
       </c>
       <c r="C42" s="37" t="n"/>
@@ -28878,37 +28898,33 @@
       <c r="E42" s="25" t="n"/>
       <c r="F42" s="25" t="n"/>
     </row>
-    <row r="44" ht="72" customFormat="1" customHeight="1" s="37">
-      <c r="C44" s="38" t="inlineStr">
-        <is>
-          <t>Doprecyzowanie po uwagach</t>
-        </is>
-      </c>
-      <c r="D44" s="39" t="inlineStr">
-        <is>
-          <t>Relacja między punktacją a kolejnością oceny</t>
-        </is>
-      </c>
-      <c r="E44" s="38" t="inlineStr">
-        <is>
-          <t>Kolejność oceny jest hierarchią merytoryczną, a punktacja jest jej technicznym odwzorowaniem. Data dokumentu jest kryterium pomocniczym stosowanym na końcu, zwłaszcza przy remisie.</t>
-        </is>
-      </c>
-    </row>
+    <row r="43">
+      <c r="A43" s="25" t="n"/>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>6. Dopiero na końcu — jaka jest data dokumentu.</t>
+        </is>
+      </c>
+      <c r="C43" s="37" t="n"/>
+      <c r="D43" s="25" t="n"/>
+      <c r="E43" s="25" t="n"/>
+      <c r="F43" s="25" t="n"/>
+    </row>
+    <row r="44" ht="72" customFormat="1" customHeight="1" s="37"/>
     <row r="45" customFormat="1" s="37">
       <c r="C45" s="38" t="inlineStr">
         <is>
-          <t>Kolejność oceny</t>
-        </is>
-      </c>
-      <c r="D45" s="38" t="inlineStr">
-        <is>
-          <t>1</t>
+          <t>Doprecyzowanie po uwagach</t>
+        </is>
+      </c>
+      <c r="D45" s="39" t="inlineStr">
+        <is>
+          <t>Relacja między punktacją a kolejnością oceny</t>
         </is>
       </c>
       <c r="E45" s="38" t="inlineStr">
         <is>
-          <t>Czy dokument dotyczy członka zarządu?</t>
+          <t>Kolejność oceny jest hierarchią merytoryczną, a punktacja jest jej technicznym odwzorowaniem. Data dokumentu jest kryterium pomocniczym stosowanym na końcu, zwłaszcza przy remisie.</t>
         </is>
       </c>
     </row>
@@ -28920,12 +28936,12 @@
       </c>
       <c r="D46" s="38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E46" s="38" t="inlineStr">
         <is>
-          <t>Czy dokument uruchamia termin na reakcję?</t>
+          <t>Czy dokument dotyczy członka zarządu?</t>
         </is>
       </c>
     </row>
@@ -28937,12 +28953,12 @@
       </c>
       <c r="D47" s="38" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E47" s="38" t="inlineStr">
         <is>
-          <t>Czy dokument dotyczy odpowiedzialności z art. 299 k.s.h. albo podobnej odpowiedzialności osoby zarządzającej?</t>
+          <t>Czy dokument uruchamia termin na reakcję?</t>
         </is>
       </c>
     </row>
@@ -28954,12 +28970,12 @@
       </c>
       <c r="D48" s="38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E48" s="38" t="inlineStr">
         <is>
-          <t>Czy dokument pochodzi z sądu, komornika albo organu publicznego?</t>
+          <t>Czy dokument dotyczy odpowiedzialności z art. 299 k.s.h. albo podobnej odpowiedzialności osoby zarządzającej?</t>
         </is>
       </c>
     </row>
@@ -28971,12 +28987,12 @@
       </c>
       <c r="D49" s="38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E49" s="38" t="inlineStr">
         <is>
-          <t>Czy dokument jest aktualny i ma bieżący termin?</t>
+          <t>Czy dokument pochodzi z sądu, komornika albo organu publicznego?</t>
         </is>
       </c>
     </row>
@@ -28988,10 +29004,27 @@
       </c>
       <c r="D50" s="38" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E50" s="38" t="inlineStr">
+        <is>
+          <t>Czy dokument jest aktualny i ma bieżący termin?</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="C51" s="38" t="inlineStr">
+        <is>
+          <t>Kolejność oceny</t>
+        </is>
+      </c>
+      <c r="D51" s="38" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E50" s="38" t="inlineStr">
+      <c r="E51" s="38" t="inlineStr">
         <is>
           <t>Dopiero na końcu — jaka jest data dokumentu.</t>
         </is>
@@ -37936,12 +37969,12 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>pozew; e-sąd; EPU; Nc-e; Sąd Rejonowy Lublin-Zachód; pozwany: członek zarządu; art. 299 ksh</t>
+          <t>pozew; P O Z E W; e-sad; EPU; Sad Rejonowy Lublin-Zachod; wartosc przedmiotu sporu; uzasadnienie; wnosimy o; wnosze o</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>pozew w elektronicznym postępowaniu upominawczym przeciwko członkowi zarządu</t>
+          <t>pozew o zaplate; powod wnosi o</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Aktualizacja CSV 04 i Excel: dodaj regule 2a, popraw regule 3 (sync z kodem)
Reguła 2a (nowa): Wśród nakazy tego samego rodzaju — nakaz z instrukcją
terminu (np. "w ciągu dwóch tygodni") wygrywa nad nakazem bez tej instrukcji.
Dokumentuje hard rule dodaną w doc_selector.py (commit d285df5).

Reguła 3 (aktualizacja): Usunięto warunek "jeżeli termin biegnie" — nakaz
ma bezwzględnie wyższy priorytet niż pozew, niezależnie od biegnącego terminu.
Dostosowanie specyfikacji do faktycznego zachowania kodu (hard rule w doc_selector.py).

Zsynchronizowane: CSV 04 ↔ arkusz 2B_Reguly_remisu w Excel.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -28807,11 +28807,7 @@
           <t>Dokument obcy tematycznie</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>Dokument nie jest dokumentem prawnym albo nie dotyczy odpowiedzialności zarządu/spółki</t>
-        </is>
-      </c>
+      <c r="C36" s="68" t="n"/>
       <c r="D36" s="5" t="n">
         <v>-100</v>
       </c>
@@ -35815,7 +35811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="9.75" customWidth="1" style="4" min="1" max="1"/>
@@ -35880,90 +35876,107 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Jeden dokument to nakaz zapłaty, drugi to pozew</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Wybrać nakaz zapłaty, jeżeli termin na sprzeciw/zarzuty jeszcze biegnie</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Oba dokumenty to nakazy tego samego rodzaju (EPU lub zwykły); jeden zawiera instrukcję terminu reakcji (np. "w ciągu dwóch tygodni"), drugi nie</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Wybrać nakaz z instrukcją terminu — strona uzasadnienia błędnie sklasyfikowana jako nakaz nie powinna wyprzedzać faktycznego nakazu EPU</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Jeden dokument pochodzi z EPU</t>
+          <t>Jeden dokument to nakaz zapłaty, drugi to pozew</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Wybrać dokument EPU, jeżeli jest skierowany do członka zarządu albo termin nadal biegnie</t>
+          <t>Wybrać nakaz zapłaty — nakaz ma bezwzględnie wyższy priorytet niż pozew niezależnie od biegnącego terminu</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Jeden dokument pochodzi od sądu, drugi od wierzyciela</t>
+          <t>Jeden dokument pochodzi z EPU</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Wybrać dokument sądowy</t>
+          <t>Wybrać dokument EPU, jeżeli jest skierowany do członka zarządu albo termin nadal biegnie</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Jeden dokument pochodzi od komornika, drugi jest wcześniejszym dokumentem wierzyciela</t>
+          <t>Jeden dokument pochodzi od sądu, drugi od wierzyciela</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Wybrać dokument komorniczy</t>
+          <t>Wybrać dokument sądowy</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Dokumenty są tego samego typu i mają podobny priorytet</t>
+          <t>Jeden dokument pochodzi od komornika, drugi jest wcześniejszym dokumentem wierzyciela</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Wybrać dokument najnowszy</t>
+          <t>Wybrać dokument komorniczy</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Dokumenty są tego samego typu i mają podobny priorytet</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Wybrać dokument najnowszy</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Nadal nie można ustalić dokumentu głównego</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Poprosić użytkownika o ręczny wybór dokumentu głównego</t>
         </is>

</xml_diff>

<commit_message>
Zsynchronizuj Excel z CSV — audyt komorka po komorce, 41/41
Audyt (03.07.2026) wykryl i naprawil rozjazdy:
- 5_Punktacja_formularza: K6_GOAL_BUY_TIME mialo w Excelu H=1 mimo
  celowej zmiany na H=0 w CSV (commit 5d0f0ba nie zsynchronizowal
  Excela) — roznica WPLYWALA na punktacje wg zrodla prawdy
- 2_Reguly_wyboru_dok_glownego: R06a mialo zdegradowane polskie znaki,
  R33 mialo scalone komorki B36:C36 i pusta kolumne Warunek
- 2B_Reguly_remisu + CSV 04: sredniki WEWNATRZ tresci komorek
  kolidowaly z separatorem CSV — zamienione na przecinek/pauze
  w obu plikach (regula 2a i 3)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -27997,22 +27997,20 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Pozew w elektronicznym postepowaniu upominawczym (EPU) przeciwko czlonkowi zarzadu</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>52</t>
-        </is>
+          <t>Pozew w elektronicznym postępowaniu upominawczym (EPU) przeciwko członkowi zarządu</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>52</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Dokument glowny - wysoki priorytet</t>
+          <t>Dokument główny — wysoki priorytet</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Jezeli sygnatura zawiera Nc-e albo wystepuje Sad Rejonowy Lublin-Zachod, dodaj flage EPU. Pozew jest wczesniejszym etapem niz nakaz - nie musi zawierac formuly nakazowej.</t>
+          <t>Jeżeli sygnatura zawiera „Nc-e" albo występuje Sąd Rejonowy Lublin-Zachód, dodaj flagę EPU. Pozew jest wcześniejszym etapem niż nakaz — nie musi zawierać formuły nakazowej.</t>
         </is>
       </c>
     </row>
@@ -28807,7 +28805,11 @@
           <t>Dokument obcy tematycznie</t>
         </is>
       </c>
-      <c r="C36" s="68" t="n"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Dokument nie jest dokumentem prawnym albo nie dotyczy odpowiedzialności zarządu/spółki</t>
+        </is>
+      </c>
       <c r="D36" s="5" t="n">
         <v>-100</v>
       </c>
@@ -29027,13 +29029,12 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="7">
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B36:C36"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B41:C41"/>
   </mergeCells>
@@ -35883,7 +35884,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Oba dokumenty to nakazy tego samego rodzaju (EPU lub zwykły); jeden zawiera instrukcję terminu reakcji (np. "w ciągu dwóch tygodni"), drugi nie</t>
+          <t>Oba dokumenty to nakazy tego samego rodzaju (EPU lub zwykły), jeden zawiera instrukcję terminu reakcji (np. "w ciągu dwóch tygodni"), drugi nie</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -35903,7 +35904,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Wybrać nakaz zapłaty — nakaz ma wyższy priorytet niż pozew niezależnie od biegnącego terminu, CHYBA ŻE nakaz dotyczy spółki, a pozew członka zarządu (sekwencja art. 299 KSH: po bezskutecznej egzekucji przeciwko spółce dokumentem wymagającym reakcji jest pozew przeciwko członkowi zarządu — nakaz jest wtedy prawomocnym dokumentem historycznym; zob. R10 w arkuszu 2). Sygnały sekwencji art. 299: w paczce jest wniosek egzekucyjny lub postanowienie o umorzeniu egzekucji, albo nakaz i pozew mają różnych pozwanych (spółka vs osoba fizyczna)</t>
+          <t>Wybrać nakaz zapłaty — nakaz ma wyższy priorytet niż pozew niezależnie od biegnącego terminu, CHYBA ŻE nakaz dotyczy spółki, a pozew członka zarządu (sekwencja art. 299 KSH: po bezskutecznej egzekucji przeciwko spółce dokumentem wymagającym reakcji jest pozew przeciwko członkowi zarządu — nakaz jest wtedy prawomocnym dokumentem historycznym — zob. R10 w arkuszu 2). Sygnały sekwencji art. 299: w paczce jest wniosek egzekucyjny lub postanowienie o umorzeniu egzekucji, albo nakaz i pozew mają różnych pozwanych (spółka vs osoba fizyczna)</t>
         </is>
       </c>
     </row>
@@ -41673,7 +41674,7 @@
         <v>0</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Popraw tresc bramki art.299 i checkboxa EPU po audycie UX formularza
Audyt pytan K1-K7 z perspektywy potencjalnego klienta wykazal, ze K2-K7 sa
napisane dobrze, ale bramka art.299 (gesty prawniczy jezyk, zero
wyjasnienia - jedyne miejsce bez "Dlaczego pytamy?") i etykieta checkboxa
EPU (zargon "sygnatura Nc-e" wprost w etykiecie) psuly pierwsze wrazenie.
Naprawione: bramka przepisana na prostszy jezyk + dodany "Dlaczego
pytamy?"; etykieta EPU skrocona (szczegoly zostaja w istniejacym,
juz dobrym expanderze).

Przy okazji: martwa kolumna question_text w CSV 08 zsynchronizowana z
realnym tekstem app.py dla K1/K4/K5/K7 (CSV+Excel). Dla K3/K6 kierunek
odwrocony na wniosek uzytkownika - realne etykiety w app.py brzmialy
niemal identycznie mimo ze pytaja o rozne rzeczy, wiec to app.py wraca
do lepszych, odroznialnych wersji z CSV.
</commit_message>
<xml_diff>
--- a/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
+++ b/dane_wejściowe/KRS_Guard_reguly_i_zasady_funkcjonowania.xlsx
@@ -42620,7 +42620,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -42667,7 +42667,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -42714,7 +42714,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -42761,7 +42761,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -42808,7 +42808,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -42855,7 +42855,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -42902,7 +42902,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -42949,7 +42949,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -42996,7 +42996,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -43513,7 +43513,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Status w zarządzie w okresie sprawy</t>
+          <t>Jaki jest Twój status w zarządzie?</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -43560,7 +43560,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Status w zarządzie w okresie sprawy</t>
+          <t>Jaki jest Twój status w zarządzie?</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -43607,7 +43607,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Status w zarządzie w okresie sprawy</t>
+          <t>Jaki jest Twój status w zarządzie?</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -43654,7 +43654,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Czy zmiana została ujawniona w KRS?</t>
+          <t>Czy zmiana w zarządzie została ujawniona w KRS?</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -43701,7 +43701,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Czy zmiana została ujawniona w KRS?</t>
+          <t>Czy zmiana w zarządzie została ujawniona w KRS?</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -43748,7 +43748,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Czy zmiana została ujawniona w KRS?</t>
+          <t>Czy zmiana w zarządzie została ujawniona w KRS?</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -43795,7 +43795,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Czy zmiana została ujawniona w KRS?</t>
+          <t>Czy zmiana w zarządzie została ujawniona w KRS?</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -44077,7 +44077,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Jaka jest kwota roszczenia wskazana w dokumencie?</t>
+          <t>Jaka kwota roszczenia jest wskazana w dokumencie?</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -44124,7 +44124,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Jaka jest kwota roszczenia wskazana w dokumencie?</t>
+          <t>Jaka kwota roszczenia jest wskazana w dokumencie?</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
@@ -44171,7 +44171,7 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Jaka jest kwota roszczenia wskazana w dokumencie?</t>
+          <t>Jaka kwota roszczenia jest wskazana w dokumencie?</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -44218,7 +44218,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Jaka jest kwota roszczenia wskazana w dokumencie?</t>
+          <t>Jaka kwota roszczenia jest wskazana w dokumencie?</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -44265,7 +44265,7 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Jaka jest kwota roszczenia wskazana w dokumencie?</t>
+          <t>Jaka kwota roszczenia jest wskazana w dokumencie?</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -44312,7 +44312,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Jaka jest kwota roszczenia wskazana w dokumencie?</t>
+          <t>Jaka kwota roszczenia jest wskazana w dokumencie?</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -44359,7 +44359,7 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
@@ -44406,7 +44406,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -44453,7 +44453,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -44500,7 +44500,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Rodzaj pisma, którego dotyczy sprawa</t>
+          <t>Jakie pismo lub dokument dotyczy Twojej sprawy?</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">

</xml_diff>